<commit_message>
Split out embedded disclaimer footers and hidden headings after review
- Footers ('The electronic version of the Senate Hansard Report ... Hansard
  Editor, Senate.') left inside blocks: split out and marked deleted, as the
  tool's Split block + X does (460 footers, 10 sittings).
- PDF headings left inside speeches where Mzalendo's wording differs from the
  PDF: split out as headings, misplaced inserted copies removed (30 headings,
  21 sittings); 11 headings broken across two blocks flagged.
- Changed sittings re-exported through the tool's Suggest hierarchy; flag
  lists renumbered. Totals now 230 finished / 189 needs check / 1,508 flags.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M7thX74TYnsQKCuCTAUqbc
</commit_message>
<xml_diff>
--- a/12th Senate - audit results/All sittings in date order - finished or needs human check.xlsx
+++ b/12th Senate - audit results/All sittings in date order - finished or needs human check.xlsx
@@ -1075,7 +1075,7 @@
         </is>
       </c>
       <c r="K16" s="6" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="L16" s="6" t="n"/>
       <c r="M16" s="6" t="n"/>
@@ -1445,7 +1445,7 @@
         </is>
       </c>
       <c r="K22" s="6" t="n">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="L22" s="6" t="n">
         <v>1</v>
@@ -1507,7 +1507,7 @@
         </is>
       </c>
       <c r="K23" s="6" t="n">
-        <v>185</v>
+        <v>260</v>
       </c>
       <c r="L23" s="6" t="n"/>
       <c r="M23" s="6" t="n"/>
@@ -1565,7 +1565,7 @@
         </is>
       </c>
       <c r="K24" s="6" t="n">
-        <v>91</v>
+        <v>185</v>
       </c>
       <c r="L24" s="6" t="n">
         <v>3</v>
@@ -1625,7 +1625,7 @@
         </is>
       </c>
       <c r="K25" s="6" t="n">
-        <v>164</v>
+        <v>250</v>
       </c>
       <c r="L25" s="6" t="n">
         <v>2</v>
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="K26" s="6" t="n">
-        <v>199</v>
+        <v>279</v>
       </c>
       <c r="L26" s="6" t="n">
         <v>34</v>
@@ -1801,7 +1801,7 @@
         </is>
       </c>
       <c r="K28" s="6" t="n">
-        <v>401</v>
+        <v>503</v>
       </c>
       <c r="L28" s="6" t="n">
         <v>6</v>
@@ -1954,7 +1954,7 @@
         </is>
       </c>
       <c r="F31" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G31" s="9" t="inlineStr">
         <is>
@@ -1986,7 +1986,9 @@
       <c r="N31" s="6" t="n"/>
       <c r="O31" s="6" t="n"/>
       <c r="P31" s="6" t="n"/>
-      <c r="Q31" s="6" t="n"/>
+      <c r="Q31" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="R31" s="10" t="inlineStr"/>
     </row>
     <row r="32">
@@ -3179,7 +3181,7 @@
         </is>
       </c>
       <c r="K52" s="6" t="n">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="L52" s="6" t="n">
         <v>1</v>
@@ -3349,7 +3351,7 @@
         </is>
       </c>
       <c r="K55" s="6" t="n">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="L55" s="6" t="n">
         <v>4</v>
@@ -3509,7 +3511,7 @@
         </is>
       </c>
       <c r="K58" s="6" t="n">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="L58" s="6" t="n"/>
       <c r="M58" s="6" t="n"/>
@@ -4520,20 +4522,24 @@
           <t>14:30</t>
         </is>
       </c>
-      <c r="E76" s="11" t="inlineStr">
-        <is>
-          <t>Finished - no issues found</t>
+      <c r="E76" s="8" t="inlineStr">
+        <is>
+          <t>Needs human check</t>
         </is>
       </c>
       <c r="F76" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G76" s="9" t="inlineStr">
         <is>
           <t>2018-07-18-14-30-00 - Senate.json</t>
         </is>
       </c>
-      <c r="H76" s="6" t="inlineStr"/>
+      <c r="H76" s="9" t="inlineStr">
+        <is>
+          <t>2018-07-18-14-30-00 - Senate - flags.txt</t>
+        </is>
+      </c>
       <c r="I76" s="6" t="inlineStr">
         <is>
           <t>2018-07-18 - Hansard Report - Wednesday, 18th July, 2018.pdf</t>
@@ -4552,7 +4558,9 @@
       <c r="N76" s="6" t="n"/>
       <c r="O76" s="6" t="n"/>
       <c r="P76" s="6" t="n"/>
-      <c r="Q76" s="6" t="n"/>
+      <c r="Q76" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="R76" s="10" t="inlineStr"/>
     </row>
     <row r="77">
@@ -4918,7 +4926,7 @@
         </is>
       </c>
       <c r="F83" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G83" s="9" t="inlineStr">
         <is>
@@ -4941,7 +4949,7 @@
         </is>
       </c>
       <c r="K83" s="6" t="n">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="L83" s="6" t="n">
         <v>3</v>
@@ -4952,7 +4960,9 @@
       <c r="N83" s="6" t="n"/>
       <c r="O83" s="6" t="n"/>
       <c r="P83" s="6" t="n"/>
-      <c r="Q83" s="6" t="n"/>
+      <c r="Q83" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="R83" s="10" t="inlineStr"/>
     </row>
     <row r="84">
@@ -5111,7 +5121,7 @@
         </is>
       </c>
       <c r="K86" s="6" t="n">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="L86" s="6" t="n">
         <v>1</v>
@@ -5383,7 +5393,7 @@
         </is>
       </c>
       <c r="K91" s="6" t="n">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="L91" s="6" t="n"/>
       <c r="M91" s="6" t="n"/>
@@ -5651,7 +5661,7 @@
         </is>
       </c>
       <c r="K96" s="6" t="n">
-        <v>210</v>
+        <v>308</v>
       </c>
       <c r="L96" s="6" t="n">
         <v>4</v>
@@ -5713,7 +5723,7 @@
         </is>
       </c>
       <c r="K97" s="6" t="n">
-        <v>443</v>
+        <v>486</v>
       </c>
       <c r="L97" s="6" t="n">
         <v>1</v>
@@ -5775,7 +5785,7 @@
         </is>
       </c>
       <c r="K98" s="6" t="n">
-        <v>176</v>
+        <v>256</v>
       </c>
       <c r="L98" s="6" t="n"/>
       <c r="M98" s="6" t="n"/>
@@ -5885,7 +5895,7 @@
         </is>
       </c>
       <c r="K100" s="6" t="n">
-        <v>271</v>
+        <v>372</v>
       </c>
       <c r="L100" s="6" t="n">
         <v>6</v>
@@ -9245,7 +9255,7 @@
         </is>
       </c>
       <c r="K160" s="6" t="n">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="L160" s="6" t="n">
         <v>2</v>
@@ -9564,7 +9574,7 @@
         </is>
       </c>
       <c r="F166" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G166" s="9" t="inlineStr">
         <is>
@@ -9598,7 +9608,9 @@
       <c r="N166" s="6" t="n"/>
       <c r="O166" s="6" t="n"/>
       <c r="P166" s="6" t="n"/>
-      <c r="Q166" s="6" t="n"/>
+      <c r="Q166" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="R166" s="10" t="inlineStr"/>
     </row>
     <row r="167">
@@ -9643,7 +9655,7 @@
         </is>
       </c>
       <c r="K167" s="6" t="n">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="L167" s="6" t="n"/>
       <c r="M167" s="6" t="n"/>
@@ -9751,7 +9763,7 @@
         </is>
       </c>
       <c r="K169" s="6" t="n">
-        <v>750</v>
+        <v>752</v>
       </c>
       <c r="L169" s="6" t="n"/>
       <c r="M169" s="6" t="n">
@@ -11812,7 +11824,7 @@
         </is>
       </c>
       <c r="F207" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G207" s="9" t="inlineStr">
         <is>
@@ -11846,7 +11858,9 @@
       <c r="N207" s="6" t="n"/>
       <c r="O207" s="6" t="n"/>
       <c r="P207" s="6" t="n"/>
-      <c r="Q207" s="6" t="n"/>
+      <c r="Q207" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="R207" s="10" t="inlineStr"/>
     </row>
     <row r="208">
@@ -14594,20 +14608,24 @@
           <t>14:30</t>
         </is>
       </c>
-      <c r="E258" s="11" t="inlineStr">
-        <is>
-          <t>Finished - no issues found</t>
+      <c r="E258" s="8" t="inlineStr">
+        <is>
+          <t>Needs human check</t>
         </is>
       </c>
       <c r="F258" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G258" s="9" t="inlineStr">
         <is>
           <t>2020-07-21-14-30-00 - Senate.json</t>
         </is>
       </c>
-      <c r="H258" s="6" t="inlineStr"/>
+      <c r="H258" s="9" t="inlineStr">
+        <is>
+          <t>2020-07-21-14-30-00 - Senate - flags.txt</t>
+        </is>
+      </c>
       <c r="I258" s="6" t="inlineStr">
         <is>
           <t>2020-07-21 - Hansard Report - Tuesday, 21st July, 2020.pdf</t>
@@ -14626,7 +14644,9 @@
       <c r="N258" s="6" t="n"/>
       <c r="O258" s="6" t="n"/>
       <c r="P258" s="6" t="n"/>
-      <c r="Q258" s="6" t="n"/>
+      <c r="Q258" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="R258" s="10" t="inlineStr"/>
     </row>
     <row r="259">
@@ -15031,7 +15051,7 @@
         </is>
       </c>
       <c r="K265" s="6" t="n">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="L265" s="6" t="n"/>
       <c r="M265" s="6" t="n"/>
@@ -15350,7 +15370,7 @@
         </is>
       </c>
       <c r="F271" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G271" s="9" t="inlineStr">
         <is>
@@ -15382,7 +15402,9 @@
       <c r="N271" s="6" t="n"/>
       <c r="O271" s="6" t="n"/>
       <c r="P271" s="6" t="n"/>
-      <c r="Q271" s="6" t="n"/>
+      <c r="Q271" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="R271" s="10" t="inlineStr"/>
     </row>
     <row r="272">
@@ -18554,20 +18576,24 @@
           <t>14:30</t>
         </is>
       </c>
-      <c r="E329" s="11" t="inlineStr">
-        <is>
-          <t>Finished - no issues found</t>
+      <c r="E329" s="8" t="inlineStr">
+        <is>
+          <t>Needs human check</t>
         </is>
       </c>
       <c r="F329" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G329" s="9" t="inlineStr">
         <is>
           <t>2021-07-07-14-30-00 - Senate.json</t>
         </is>
       </c>
-      <c r="H329" s="6" t="inlineStr"/>
+      <c r="H329" s="9" t="inlineStr">
+        <is>
+          <t>2021-07-07-14-30-00 - Senate - flags.txt</t>
+        </is>
+      </c>
       <c r="I329" s="6" t="inlineStr">
         <is>
           <t>2021-07-07 - Hansard Report - Wednesday, 7th July, 2021.pdf</t>
@@ -18586,7 +18612,9 @@
       <c r="N329" s="6" t="n"/>
       <c r="O329" s="6" t="n"/>
       <c r="P329" s="6" t="n"/>
-      <c r="Q329" s="6" t="n"/>
+      <c r="Q329" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="R329" s="10" t="inlineStr"/>
     </row>
     <row r="330">
@@ -23568,7 +23596,7 @@
         </is>
       </c>
       <c r="F423" s="6" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G423" s="9" t="inlineStr">
         <is>
@@ -23602,7 +23630,9 @@
       </c>
       <c r="O423" s="6" t="n"/>
       <c r="P423" s="6" t="n"/>
-      <c r="Q423" s="6" t="n"/>
+      <c r="Q423" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="R423" s="10" t="inlineStr"/>
     </row>
     <row r="424">
@@ -24074,856 +24104,859 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G75" r:id="rId176"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J75" r:id="rId177"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G76" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J76" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G77" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J77" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G78" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J78" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G79" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H79" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J79" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G80" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H80" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J80" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G81" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H81" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J81" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G82" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H82" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J82" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G83" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H83" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J83" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G84" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H84" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J84" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G85" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J85" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G86" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H86" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J86" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G87" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J87" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G88" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J88" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G89" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H89" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J89" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G90" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J90" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G91" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J91" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G92" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H92" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J92" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G93" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H93" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J93" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G94" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J94" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G95" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J95" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G96" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H96" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J96" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G97" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H97" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J97" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G98" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H98" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J98" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G99" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J99" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G100" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H100" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J100" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G101" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H101" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J101" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G102" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H102" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J102" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G103" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H103" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J103" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G104" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J104" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G105" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J105" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G106" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J106" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G107" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J107" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G108" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J108" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G109" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J109" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G110" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H110" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J110" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G111" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J111" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G112" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J112" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G113" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J113" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G114" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H114" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J114" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G115" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H115" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J115" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G116" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H116" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J116" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G117" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H117" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J117" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G118" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J118" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G119" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J119" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G120" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H120" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J120" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G121" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H121" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J121" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G122" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J122" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G123" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J123" r:id="rId297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G124" r:id="rId298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H124" r:id="rId299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J124" r:id="rId300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G125" r:id="rId301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H125" r:id="rId302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J125" r:id="rId303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G126" r:id="rId304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H126" r:id="rId305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J126" r:id="rId306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G127" r:id="rId307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H127" r:id="rId308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J127" r:id="rId309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G128" r:id="rId310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J128" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G129" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H129" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J129" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G130" r:id="rId315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H130" r:id="rId316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J130" r:id="rId317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G131" r:id="rId318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H131" r:id="rId319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J131" r:id="rId320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G132" r:id="rId321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J132" r:id="rId322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G133" r:id="rId323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J133" r:id="rId324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G134" r:id="rId325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J134" r:id="rId326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G135" r:id="rId327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H135" r:id="rId328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J135" r:id="rId329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G136" r:id="rId330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H136" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J136" r:id="rId332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G137" r:id="rId333"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J137" r:id="rId334"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G138" r:id="rId335"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J138" r:id="rId336"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G139" r:id="rId337"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J139" r:id="rId338"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G140" r:id="rId339"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H140" r:id="rId340"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J140" r:id="rId341"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G141" r:id="rId342"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H141" r:id="rId343"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J141" r:id="rId344"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G142" r:id="rId345"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J142" r:id="rId346"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G143" r:id="rId347"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H143" r:id="rId348"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J143" r:id="rId349"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G144" r:id="rId350"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H144" r:id="rId351"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J144" r:id="rId352"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G145" r:id="rId353"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J145" r:id="rId354"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G146" r:id="rId355"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H146" r:id="rId356"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J146" r:id="rId357"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G147" r:id="rId358"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J147" r:id="rId359"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G148" r:id="rId360"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J148" r:id="rId361"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G149" r:id="rId362"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H149" r:id="rId363"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J149" r:id="rId364"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G150" r:id="rId365"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J150" r:id="rId366"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G151" r:id="rId367"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J151" r:id="rId368"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G152" r:id="rId369"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H152" r:id="rId370"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J152" r:id="rId371"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G153" r:id="rId372"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H153" r:id="rId373"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J153" r:id="rId374"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G154" r:id="rId375"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H154" r:id="rId376"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J154" r:id="rId377"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G155" r:id="rId378"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J155" r:id="rId379"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G156" r:id="rId380"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H156" r:id="rId381"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J156" r:id="rId382"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G157" r:id="rId383"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J157" r:id="rId384"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G158" r:id="rId385"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J158" r:id="rId386"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G159" r:id="rId387"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H159" r:id="rId388"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J159" r:id="rId389"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G160" r:id="rId390"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H160" r:id="rId391"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J160" r:id="rId392"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G161" r:id="rId393"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H161" r:id="rId394"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J161" r:id="rId395"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G162" r:id="rId396"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H162" r:id="rId397"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J162" r:id="rId398"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G163" r:id="rId399"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J163" r:id="rId400"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G164" r:id="rId401"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H164" r:id="rId402"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J164" r:id="rId403"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G165" r:id="rId404"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J165" r:id="rId405"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G166" r:id="rId406"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H166" r:id="rId407"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J166" r:id="rId408"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G167" r:id="rId409"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J167" r:id="rId410"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G168" r:id="rId411"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J168" r:id="rId412"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G169" r:id="rId413"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H169" r:id="rId414"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J169" r:id="rId415"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G170" r:id="rId416"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H170" r:id="rId417"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J170" r:id="rId418"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G171" r:id="rId419"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H171" r:id="rId420"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J171" r:id="rId421"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G172" r:id="rId422"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J172" r:id="rId423"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G173" r:id="rId424"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H173" r:id="rId425"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J173" r:id="rId426"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G174" r:id="rId427"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H174" r:id="rId428"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J174" r:id="rId429"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G175" r:id="rId430"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H175" r:id="rId431"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J175" r:id="rId432"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G176" r:id="rId433"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H176" r:id="rId434"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J176" r:id="rId435"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G177" r:id="rId436"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J177" r:id="rId437"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G178" r:id="rId438"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H178" r:id="rId439"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J178" r:id="rId440"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G179" r:id="rId441"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H179" r:id="rId442"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J179" r:id="rId443"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G180" r:id="rId444"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H180" r:id="rId445"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J180" r:id="rId446"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G181" r:id="rId447"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J181" r:id="rId448"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G182" r:id="rId449"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J182" r:id="rId450"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G183" r:id="rId451"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H183" r:id="rId452"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J183" r:id="rId453"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G184" r:id="rId454"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H184" r:id="rId455"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J184" r:id="rId456"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G185" r:id="rId457"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J185" r:id="rId458"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G186" r:id="rId459"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H186" r:id="rId460"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J186" r:id="rId461"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G187" r:id="rId462"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H187" r:id="rId463"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J187" r:id="rId464"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G188" r:id="rId465"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J188" r:id="rId466"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G189" r:id="rId467"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H189" r:id="rId468"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J189" r:id="rId469"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G190" r:id="rId470"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J190" r:id="rId471"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G191" r:id="rId472"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J191" r:id="rId473"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G192" r:id="rId474"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H192" r:id="rId475"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J192" r:id="rId476"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G193" r:id="rId477"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J193" r:id="rId478"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G194" r:id="rId479"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J194" r:id="rId480"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G195" r:id="rId481"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J195" r:id="rId482"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G196" r:id="rId483"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J196" r:id="rId484"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G197" r:id="rId485"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H197" r:id="rId486"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J197" r:id="rId487"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G198" r:id="rId488"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J198" r:id="rId489"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G199" r:id="rId490"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J199" r:id="rId491"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G200" r:id="rId492"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J200" r:id="rId493"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G201" r:id="rId494"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J201" r:id="rId495"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G202" r:id="rId496"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J202" r:id="rId497"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G203" r:id="rId498"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J203" r:id="rId499"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G204" r:id="rId500"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J204" r:id="rId501"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G205" r:id="rId502"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J205" r:id="rId503"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G206" r:id="rId504"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J206" r:id="rId505"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G207" r:id="rId506"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H207" r:id="rId507"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J207" r:id="rId508"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G208" r:id="rId509"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J208" r:id="rId510"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G209" r:id="rId511"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H209" r:id="rId512"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J209" r:id="rId513"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G210" r:id="rId514"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J210" r:id="rId515"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G211" r:id="rId516"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J211" r:id="rId517"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G212" r:id="rId518"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J212" r:id="rId519"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G213" r:id="rId520"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J213" r:id="rId521"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G214" r:id="rId522"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J214" r:id="rId523"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G215" r:id="rId524"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J215" r:id="rId525"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G216" r:id="rId526"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H216" r:id="rId527"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J216" r:id="rId528"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G217" r:id="rId529"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J217" r:id="rId530"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G218" r:id="rId531"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H218" r:id="rId532"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J218" r:id="rId533"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G219" r:id="rId534"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H219" r:id="rId535"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J219" r:id="rId536"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G220" r:id="rId537"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J220" r:id="rId538"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G221" r:id="rId539"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J221" r:id="rId540"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G222" r:id="rId541"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H222" r:id="rId542"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J222" r:id="rId543"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G223" r:id="rId544"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J223" r:id="rId545"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G224" r:id="rId546"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J224" r:id="rId547"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G225" r:id="rId548"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H225" r:id="rId549"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J225" r:id="rId550"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G226" r:id="rId551"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J226" r:id="rId552"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G227" r:id="rId553"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J227" r:id="rId554"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G228" r:id="rId555"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J228" r:id="rId556"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G229" r:id="rId557"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J229" r:id="rId558"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G230" r:id="rId559"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J230" r:id="rId560"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G231" r:id="rId561"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J231" r:id="rId562"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G232" r:id="rId563"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H232" r:id="rId564"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J232" r:id="rId565"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G233" r:id="rId566"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J233" r:id="rId567"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G234" r:id="rId568"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J234" r:id="rId569"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G235" r:id="rId570"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J235" r:id="rId571"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G236" r:id="rId572"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H236" r:id="rId573"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J236" r:id="rId574"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G237" r:id="rId575"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J237" r:id="rId576"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G238" r:id="rId577"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J238" r:id="rId578"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G239" r:id="rId579"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H239" r:id="rId580"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J239" r:id="rId581"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G240" r:id="rId582"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H240" r:id="rId583"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J240" r:id="rId584"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G241" r:id="rId585"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J241" r:id="rId586"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G242" r:id="rId587"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H242" r:id="rId588"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J242" r:id="rId589"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G243" r:id="rId590"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J243" r:id="rId591"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G244" r:id="rId592"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H244" r:id="rId593"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J244" r:id="rId594"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G245" r:id="rId595"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J245" r:id="rId596"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G246" r:id="rId597"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J246" r:id="rId598"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G247" r:id="rId599"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J247" r:id="rId600"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G248" r:id="rId601"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J248" r:id="rId602"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G249" r:id="rId603"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H249" r:id="rId604"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J249" r:id="rId605"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G250" r:id="rId606"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J250" r:id="rId607"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G251" r:id="rId608"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H251" r:id="rId609"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J251" r:id="rId610"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G252" r:id="rId611"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J252" r:id="rId612"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G253" r:id="rId613"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J253" r:id="rId614"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G254" r:id="rId615"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H254" r:id="rId616"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J254" r:id="rId617"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G255" r:id="rId618"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H255" r:id="rId619"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J255" r:id="rId620"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G256" r:id="rId621"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J256" r:id="rId622"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G257" r:id="rId623"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J257" r:id="rId624"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G258" r:id="rId625"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J258" r:id="rId626"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G259" r:id="rId627"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H259" r:id="rId628"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J259" r:id="rId629"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G260" r:id="rId630"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H260" r:id="rId631"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J260" r:id="rId632"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G261" r:id="rId633"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H261" r:id="rId634"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J261" r:id="rId635"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G262" r:id="rId636"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H262" r:id="rId637"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J262" r:id="rId638"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G263" r:id="rId639"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H263" r:id="rId640"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J263" r:id="rId641"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G264" r:id="rId642"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H264" r:id="rId643"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J264" r:id="rId644"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G265" r:id="rId645"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J265" r:id="rId646"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G266" r:id="rId647"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J266" r:id="rId648"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G267" r:id="rId649"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H267" r:id="rId650"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J267" r:id="rId651"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G268" r:id="rId652"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H268" r:id="rId653"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J268" r:id="rId654"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G269" r:id="rId655"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H269" r:id="rId656"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J269" r:id="rId657"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G270" r:id="rId658"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H270" r:id="rId659"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J270" r:id="rId660"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G271" r:id="rId661"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H271" r:id="rId662"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J271" r:id="rId663"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G272" r:id="rId664"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H272" r:id="rId665"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J272" r:id="rId666"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G273" r:id="rId667"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J273" r:id="rId668"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G274" r:id="rId669"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H274" r:id="rId670"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J274" r:id="rId671"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G275" r:id="rId672"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J275" r:id="rId673"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G276" r:id="rId674"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J276" r:id="rId675"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G277" r:id="rId676"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J277" r:id="rId677"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G278" r:id="rId678"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H278" r:id="rId679"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J278" r:id="rId680"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G279" r:id="rId681"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H279" r:id="rId682"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J279" r:id="rId683"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G280" r:id="rId684"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H280" r:id="rId685"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J280" r:id="rId686"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G281" r:id="rId687"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J281" r:id="rId688"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G282" r:id="rId689"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H282" r:id="rId690"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J282" r:id="rId691"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G283" r:id="rId692"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J283" r:id="rId693"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G284" r:id="rId694"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H284" r:id="rId695"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J284" r:id="rId696"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G285" r:id="rId697"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J285" r:id="rId698"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G286" r:id="rId699"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H286" r:id="rId700"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J286" r:id="rId701"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G287" r:id="rId702"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J287" r:id="rId703"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G288" r:id="rId704"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H288" r:id="rId705"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J288" r:id="rId706"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G289" r:id="rId707"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H289" r:id="rId708"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J289" r:id="rId709"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G290" r:id="rId710"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H290" r:id="rId711"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J290" r:id="rId712"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G291" r:id="rId713"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H291" r:id="rId714"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J291" r:id="rId715"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G292" r:id="rId716"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J292" r:id="rId717"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G293" r:id="rId718"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J293" r:id="rId719"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G294" r:id="rId720"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J294" r:id="rId721"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G295" r:id="rId722"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H295" r:id="rId723"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J295" r:id="rId724"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G296" r:id="rId725"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J296" r:id="rId726"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G297" r:id="rId727"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H297" r:id="rId728"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J297" r:id="rId729"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G298" r:id="rId730"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J298" r:id="rId731"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G299" r:id="rId732"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J299" r:id="rId733"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G300" r:id="rId734"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H300" r:id="rId735"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J300" r:id="rId736"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G301" r:id="rId737"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H301" r:id="rId738"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J301" r:id="rId739"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G302" r:id="rId740"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J302" r:id="rId741"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G303" r:id="rId742"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J303" r:id="rId743"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G304" r:id="rId744"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J304" r:id="rId745"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G305" r:id="rId746"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J305" r:id="rId747"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G306" r:id="rId748"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H306" r:id="rId749"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J306" r:id="rId750"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G307" r:id="rId751"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J307" r:id="rId752"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G308" r:id="rId753"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H308" r:id="rId754"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J308" r:id="rId755"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G309" r:id="rId756"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J309" r:id="rId757"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G310" r:id="rId758"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J310" r:id="rId759"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G311" r:id="rId760"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J311" r:id="rId761"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G312" r:id="rId762"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J312" r:id="rId763"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G313" r:id="rId764"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J313" r:id="rId765"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G314" r:id="rId766"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J314" r:id="rId767"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G315" r:id="rId768"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J315" r:id="rId769"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G316" r:id="rId770"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J316" r:id="rId771"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G317" r:id="rId772"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J317" r:id="rId773"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G318" r:id="rId774"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J318" r:id="rId775"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G319" r:id="rId776"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H319" r:id="rId777"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J319" r:id="rId778"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G320" r:id="rId779"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H320" r:id="rId780"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J320" r:id="rId781"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G321" r:id="rId782"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J321" r:id="rId783"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G322" r:id="rId784"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J322" r:id="rId785"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G323" r:id="rId786"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J323" r:id="rId787"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G324" r:id="rId788"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H324" r:id="rId789"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J324" r:id="rId790"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G325" r:id="rId791"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H325" r:id="rId792"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J325" r:id="rId793"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G326" r:id="rId794"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J326" r:id="rId795"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G327" r:id="rId796"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J327" r:id="rId797"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G328" r:id="rId798"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H328" r:id="rId799"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J328" r:id="rId800"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G329" r:id="rId801"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J329" r:id="rId802"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G330" r:id="rId803"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J330" r:id="rId804"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G331" r:id="rId805"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J331" r:id="rId806"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G332" r:id="rId807"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J332" r:id="rId808"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G333" r:id="rId809"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J333" r:id="rId810"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G334" r:id="rId811"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J334" r:id="rId812"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G335" r:id="rId813"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J335" r:id="rId814"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G336" r:id="rId815"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J336" r:id="rId816"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G337" r:id="rId817"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J337" r:id="rId818"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G338" r:id="rId819"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H338" r:id="rId820"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J338" r:id="rId821"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G339" r:id="rId822"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H339" r:id="rId823"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J339" r:id="rId824"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G340" r:id="rId825"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H340" r:id="rId826"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J340" r:id="rId827"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G341" r:id="rId828"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H341" r:id="rId829"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J341" r:id="rId830"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G342" r:id="rId831"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J342" r:id="rId832"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G343" r:id="rId833"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J343" r:id="rId834"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G344" r:id="rId835"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H344" r:id="rId836"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J344" r:id="rId837"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G345" r:id="rId838"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H345" r:id="rId839"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J345" r:id="rId840"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G346" r:id="rId841"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J346" r:id="rId842"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G347" r:id="rId843"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J347" r:id="rId844"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G348" r:id="rId845"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J348" r:id="rId846"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G349" r:id="rId847"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J349" r:id="rId848"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G350" r:id="rId849"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H350" r:id="rId850"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J350" r:id="rId851"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G351" r:id="rId852"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J351" r:id="rId853"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G352" r:id="rId854"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J352" r:id="rId855"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G353" r:id="rId856"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H353" r:id="rId857"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J353" r:id="rId858"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G354" r:id="rId859"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J354" r:id="rId860"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G355" r:id="rId861"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J355" r:id="rId862"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G356" r:id="rId863"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J356" r:id="rId864"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G357" r:id="rId865"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J357" r:id="rId866"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G358" r:id="rId867"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J358" r:id="rId868"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G359" r:id="rId869"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J359" r:id="rId870"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G360" r:id="rId871"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J360" r:id="rId872"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G361" r:id="rId873"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H361" r:id="rId874"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J361" r:id="rId875"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G362" r:id="rId876"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J362" r:id="rId877"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G363" r:id="rId878"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J363" r:id="rId879"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G364" r:id="rId880"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J364" r:id="rId881"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G365" r:id="rId882"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J365" r:id="rId883"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G366" r:id="rId884"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J366" r:id="rId885"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G367" r:id="rId886"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J367" r:id="rId887"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G368" r:id="rId888"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J368" r:id="rId889"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G369" r:id="rId890"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J369" r:id="rId891"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G370" r:id="rId892"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J370" r:id="rId893"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G371" r:id="rId894"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J371" r:id="rId895"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G372" r:id="rId896"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J372" r:id="rId897"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G373" r:id="rId898"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J373" r:id="rId899"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G374" r:id="rId900"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H374" r:id="rId901"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J374" r:id="rId902"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G375" r:id="rId903"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J375" r:id="rId904"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G376" r:id="rId905"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J376" r:id="rId906"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G377" r:id="rId907"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J377" r:id="rId908"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G378" r:id="rId909"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J378" r:id="rId910"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G379" r:id="rId911"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J379" r:id="rId912"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G380" r:id="rId913"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H380" r:id="rId914"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J380" r:id="rId915"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G381" r:id="rId916"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J381" r:id="rId917"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G382" r:id="rId918"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J382" r:id="rId919"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G383" r:id="rId920"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J383" r:id="rId921"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G384" r:id="rId922"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H384" r:id="rId923"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J384" r:id="rId924"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G385" r:id="rId925"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J385" r:id="rId926"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G386" r:id="rId927"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J386" r:id="rId928"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G387" r:id="rId929"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J387" r:id="rId930"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G388" r:id="rId931"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J388" r:id="rId932"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G389" r:id="rId933"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J389" r:id="rId934"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G390" r:id="rId935"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J390" r:id="rId936"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G391" r:id="rId937"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J391" r:id="rId938"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G392" r:id="rId939"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J392" r:id="rId940"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G393" r:id="rId941"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J393" r:id="rId942"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G394" r:id="rId943"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J394" r:id="rId944"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G395" r:id="rId945"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J395" r:id="rId946"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G396" r:id="rId947"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J396" r:id="rId948"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G397" r:id="rId949"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H397" r:id="rId950"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J397" r:id="rId951"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G398" r:id="rId952"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J398" r:id="rId953"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G399" r:id="rId954"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H399" r:id="rId955"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J399" r:id="rId956"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G400" r:id="rId957"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J400" r:id="rId958"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G401" r:id="rId959"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H401" r:id="rId960"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J401" r:id="rId961"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G402" r:id="rId962"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H402" r:id="rId963"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J402" r:id="rId964"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G403" r:id="rId965"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J403" r:id="rId966"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G404" r:id="rId967"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J404" r:id="rId968"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G405" r:id="rId969"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J405" r:id="rId970"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G406" r:id="rId971"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H406" r:id="rId972"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J406" r:id="rId973"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G407" r:id="rId974"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H407" r:id="rId975"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J407" r:id="rId976"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G408" r:id="rId977"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J408" r:id="rId978"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G409" r:id="rId979"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H409" r:id="rId980"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J409" r:id="rId981"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G410" r:id="rId982"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J410" r:id="rId983"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G411" r:id="rId984"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J411" r:id="rId985"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G412" r:id="rId986"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J412" r:id="rId987"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G413" r:id="rId988"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J413" r:id="rId989"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G414" r:id="rId990"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J414" r:id="rId991"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G415" r:id="rId992"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J415" r:id="rId993"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G416" r:id="rId994"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J416" r:id="rId995"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G417" r:id="rId996"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J417" r:id="rId997"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G418" r:id="rId998"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J418" r:id="rId999"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G419" r:id="rId1000"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J419" r:id="rId1001"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G420" r:id="rId1002"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J420" r:id="rId1003"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G421" r:id="rId1004"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J421" r:id="rId1005"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G422" r:id="rId1006"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H422" r:id="rId1007"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J422" r:id="rId1008"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G423" r:id="rId1009"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H423" r:id="rId1010"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J423" r:id="rId1011"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G424" r:id="rId1012"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H424" r:id="rId1013"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J424" r:id="rId1014"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G425" r:id="rId1015"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H425" r:id="rId1016"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J425" r:id="rId1017"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G426" r:id="rId1018"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J426" r:id="rId1019"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G427" r:id="rId1020"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H427" r:id="rId1021"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J427" r:id="rId1022"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G428" r:id="rId1023"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J428" r:id="rId1024"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J76" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G77" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J77" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G78" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J78" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G79" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H79" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J79" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G80" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H80" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J80" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G81" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H81" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J81" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G82" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H82" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J82" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G83" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H83" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J83" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G84" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H84" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J84" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G85" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J85" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G86" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H86" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J86" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G87" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J87" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G88" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J88" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G89" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H89" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J89" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G90" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J90" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G91" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J91" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G92" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H92" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J92" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G93" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H93" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J93" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G94" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J94" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G95" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J95" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G96" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H96" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J96" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G97" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H97" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J97" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G98" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H98" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J98" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G99" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J99" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G100" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H100" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J100" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G101" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H101" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J101" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G102" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H102" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J102" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G103" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H103" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J103" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G104" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J104" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G105" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J105" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G106" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J106" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G107" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J107" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G108" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J108" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G109" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J109" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G110" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H110" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J110" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G111" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J111" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G112" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J112" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G113" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J113" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G114" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H114" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J114" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G115" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H115" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J115" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G116" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H116" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J116" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G117" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H117" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J117" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G118" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J118" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G119" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J119" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G120" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H120" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J120" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G121" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H121" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J121" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G122" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J122" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G123" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J123" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G124" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H124" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J124" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G125" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H125" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J125" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G126" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H126" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J126" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G127" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H127" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J127" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G128" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J128" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G129" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H129" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J129" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G130" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H130" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J130" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G131" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H131" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J131" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G132" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J132" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G133" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J133" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G134" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J134" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G135" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H135" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J135" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G136" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H136" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J136" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G137" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J137" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G138" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J138" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G139" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J139" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G140" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H140" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J140" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G141" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H141" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J141" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G142" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J142" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G143" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H143" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J143" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G144" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H144" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J144" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G145" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J145" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G146" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H146" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J146" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G147" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J147" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G148" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J148" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G149" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H149" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J149" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G150" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J150" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G151" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J151" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G152" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H152" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J152" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G153" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H153" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J153" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G154" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H154" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J154" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G155" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J155" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G156" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H156" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J156" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G157" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J157" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G158" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J158" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G159" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H159" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J159" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G160" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H160" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J160" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G161" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H161" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J161" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G162" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H162" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J162" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G163" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J163" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G164" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H164" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J164" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G165" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J165" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G166" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H166" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J166" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G167" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J167" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G168" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J168" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G169" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H169" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J169" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G170" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H170" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J170" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G171" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H171" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J171" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G172" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J172" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G173" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H173" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J173" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G174" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H174" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J174" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G175" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H175" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J175" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G176" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H176" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J176" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G177" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J177" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G178" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H178" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J178" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G179" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H179" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J179" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G180" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H180" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J180" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G181" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J181" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G182" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J182" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G183" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H183" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J183" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G184" r:id="rId455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H184" r:id="rId456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J184" r:id="rId457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G185" r:id="rId458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J185" r:id="rId459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G186" r:id="rId460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H186" r:id="rId461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J186" r:id="rId462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G187" r:id="rId463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H187" r:id="rId464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J187" r:id="rId465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G188" r:id="rId466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J188" r:id="rId467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G189" r:id="rId468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H189" r:id="rId469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J189" r:id="rId470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G190" r:id="rId471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J190" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G191" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J191" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G192" r:id="rId475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H192" r:id="rId476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J192" r:id="rId477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G193" r:id="rId478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J193" r:id="rId479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G194" r:id="rId480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J194" r:id="rId481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G195" r:id="rId482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J195" r:id="rId483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G196" r:id="rId484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J196" r:id="rId485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G197" r:id="rId486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H197" r:id="rId487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J197" r:id="rId488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G198" r:id="rId489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J198" r:id="rId490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G199" r:id="rId491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J199" r:id="rId492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G200" r:id="rId493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J200" r:id="rId494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G201" r:id="rId495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J201" r:id="rId496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G202" r:id="rId497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J202" r:id="rId498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G203" r:id="rId499"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J203" r:id="rId500"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G204" r:id="rId501"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J204" r:id="rId502"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G205" r:id="rId503"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J205" r:id="rId504"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G206" r:id="rId505"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J206" r:id="rId506"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G207" r:id="rId507"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H207" r:id="rId508"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J207" r:id="rId509"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G208" r:id="rId510"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J208" r:id="rId511"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G209" r:id="rId512"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H209" r:id="rId513"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J209" r:id="rId514"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G210" r:id="rId515"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J210" r:id="rId516"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G211" r:id="rId517"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J211" r:id="rId518"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G212" r:id="rId519"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J212" r:id="rId520"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G213" r:id="rId521"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J213" r:id="rId522"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G214" r:id="rId523"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J214" r:id="rId524"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G215" r:id="rId525"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J215" r:id="rId526"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G216" r:id="rId527"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H216" r:id="rId528"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J216" r:id="rId529"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G217" r:id="rId530"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J217" r:id="rId531"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G218" r:id="rId532"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H218" r:id="rId533"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J218" r:id="rId534"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G219" r:id="rId535"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H219" r:id="rId536"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J219" r:id="rId537"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G220" r:id="rId538"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J220" r:id="rId539"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G221" r:id="rId540"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J221" r:id="rId541"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G222" r:id="rId542"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H222" r:id="rId543"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J222" r:id="rId544"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G223" r:id="rId545"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J223" r:id="rId546"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G224" r:id="rId547"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J224" r:id="rId548"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G225" r:id="rId549"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H225" r:id="rId550"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J225" r:id="rId551"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G226" r:id="rId552"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J226" r:id="rId553"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G227" r:id="rId554"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J227" r:id="rId555"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G228" r:id="rId556"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J228" r:id="rId557"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G229" r:id="rId558"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J229" r:id="rId559"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G230" r:id="rId560"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J230" r:id="rId561"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G231" r:id="rId562"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J231" r:id="rId563"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G232" r:id="rId564"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H232" r:id="rId565"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J232" r:id="rId566"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G233" r:id="rId567"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J233" r:id="rId568"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G234" r:id="rId569"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J234" r:id="rId570"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G235" r:id="rId571"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J235" r:id="rId572"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G236" r:id="rId573"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H236" r:id="rId574"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J236" r:id="rId575"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G237" r:id="rId576"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J237" r:id="rId577"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G238" r:id="rId578"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J238" r:id="rId579"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G239" r:id="rId580"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H239" r:id="rId581"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J239" r:id="rId582"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G240" r:id="rId583"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H240" r:id="rId584"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J240" r:id="rId585"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G241" r:id="rId586"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J241" r:id="rId587"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G242" r:id="rId588"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H242" r:id="rId589"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J242" r:id="rId590"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G243" r:id="rId591"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J243" r:id="rId592"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G244" r:id="rId593"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H244" r:id="rId594"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J244" r:id="rId595"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G245" r:id="rId596"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J245" r:id="rId597"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G246" r:id="rId598"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J246" r:id="rId599"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G247" r:id="rId600"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J247" r:id="rId601"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G248" r:id="rId602"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J248" r:id="rId603"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G249" r:id="rId604"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H249" r:id="rId605"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J249" r:id="rId606"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G250" r:id="rId607"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J250" r:id="rId608"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G251" r:id="rId609"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H251" r:id="rId610"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J251" r:id="rId611"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G252" r:id="rId612"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J252" r:id="rId613"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G253" r:id="rId614"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J253" r:id="rId615"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G254" r:id="rId616"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H254" r:id="rId617"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J254" r:id="rId618"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G255" r:id="rId619"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H255" r:id="rId620"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J255" r:id="rId621"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G256" r:id="rId622"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J256" r:id="rId623"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G257" r:id="rId624"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J257" r:id="rId625"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G258" r:id="rId626"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H258" r:id="rId627"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J258" r:id="rId628"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G259" r:id="rId629"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H259" r:id="rId630"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J259" r:id="rId631"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G260" r:id="rId632"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H260" r:id="rId633"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J260" r:id="rId634"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G261" r:id="rId635"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H261" r:id="rId636"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J261" r:id="rId637"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G262" r:id="rId638"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H262" r:id="rId639"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J262" r:id="rId640"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G263" r:id="rId641"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H263" r:id="rId642"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J263" r:id="rId643"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G264" r:id="rId644"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H264" r:id="rId645"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J264" r:id="rId646"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G265" r:id="rId647"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J265" r:id="rId648"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G266" r:id="rId649"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J266" r:id="rId650"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G267" r:id="rId651"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H267" r:id="rId652"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J267" r:id="rId653"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G268" r:id="rId654"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H268" r:id="rId655"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J268" r:id="rId656"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G269" r:id="rId657"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H269" r:id="rId658"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J269" r:id="rId659"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G270" r:id="rId660"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H270" r:id="rId661"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J270" r:id="rId662"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G271" r:id="rId663"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H271" r:id="rId664"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J271" r:id="rId665"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G272" r:id="rId666"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H272" r:id="rId667"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J272" r:id="rId668"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G273" r:id="rId669"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J273" r:id="rId670"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G274" r:id="rId671"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H274" r:id="rId672"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J274" r:id="rId673"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G275" r:id="rId674"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J275" r:id="rId675"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G276" r:id="rId676"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J276" r:id="rId677"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G277" r:id="rId678"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J277" r:id="rId679"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G278" r:id="rId680"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H278" r:id="rId681"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J278" r:id="rId682"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G279" r:id="rId683"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H279" r:id="rId684"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J279" r:id="rId685"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G280" r:id="rId686"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H280" r:id="rId687"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J280" r:id="rId688"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G281" r:id="rId689"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J281" r:id="rId690"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G282" r:id="rId691"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H282" r:id="rId692"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J282" r:id="rId693"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G283" r:id="rId694"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J283" r:id="rId695"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G284" r:id="rId696"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H284" r:id="rId697"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J284" r:id="rId698"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G285" r:id="rId699"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J285" r:id="rId700"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G286" r:id="rId701"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H286" r:id="rId702"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J286" r:id="rId703"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G287" r:id="rId704"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J287" r:id="rId705"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G288" r:id="rId706"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H288" r:id="rId707"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J288" r:id="rId708"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G289" r:id="rId709"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H289" r:id="rId710"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J289" r:id="rId711"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G290" r:id="rId712"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H290" r:id="rId713"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J290" r:id="rId714"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G291" r:id="rId715"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H291" r:id="rId716"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J291" r:id="rId717"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G292" r:id="rId718"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J292" r:id="rId719"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G293" r:id="rId720"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J293" r:id="rId721"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G294" r:id="rId722"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J294" r:id="rId723"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G295" r:id="rId724"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H295" r:id="rId725"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J295" r:id="rId726"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G296" r:id="rId727"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J296" r:id="rId728"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G297" r:id="rId729"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H297" r:id="rId730"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J297" r:id="rId731"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G298" r:id="rId732"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J298" r:id="rId733"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G299" r:id="rId734"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J299" r:id="rId735"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G300" r:id="rId736"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H300" r:id="rId737"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J300" r:id="rId738"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G301" r:id="rId739"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H301" r:id="rId740"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J301" r:id="rId741"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G302" r:id="rId742"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J302" r:id="rId743"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G303" r:id="rId744"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J303" r:id="rId745"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G304" r:id="rId746"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J304" r:id="rId747"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G305" r:id="rId748"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J305" r:id="rId749"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G306" r:id="rId750"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H306" r:id="rId751"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J306" r:id="rId752"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G307" r:id="rId753"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J307" r:id="rId754"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G308" r:id="rId755"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H308" r:id="rId756"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J308" r:id="rId757"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G309" r:id="rId758"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J309" r:id="rId759"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G310" r:id="rId760"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J310" r:id="rId761"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G311" r:id="rId762"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J311" r:id="rId763"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G312" r:id="rId764"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J312" r:id="rId765"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G313" r:id="rId766"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J313" r:id="rId767"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G314" r:id="rId768"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J314" r:id="rId769"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G315" r:id="rId770"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J315" r:id="rId771"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G316" r:id="rId772"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J316" r:id="rId773"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G317" r:id="rId774"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J317" r:id="rId775"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G318" r:id="rId776"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J318" r:id="rId777"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G319" r:id="rId778"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H319" r:id="rId779"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J319" r:id="rId780"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G320" r:id="rId781"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H320" r:id="rId782"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J320" r:id="rId783"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G321" r:id="rId784"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J321" r:id="rId785"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G322" r:id="rId786"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J322" r:id="rId787"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G323" r:id="rId788"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J323" r:id="rId789"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G324" r:id="rId790"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H324" r:id="rId791"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J324" r:id="rId792"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G325" r:id="rId793"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H325" r:id="rId794"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J325" r:id="rId795"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G326" r:id="rId796"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J326" r:id="rId797"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G327" r:id="rId798"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J327" r:id="rId799"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G328" r:id="rId800"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H328" r:id="rId801"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J328" r:id="rId802"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G329" r:id="rId803"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H329" r:id="rId804"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J329" r:id="rId805"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G330" r:id="rId806"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J330" r:id="rId807"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G331" r:id="rId808"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J331" r:id="rId809"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G332" r:id="rId810"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J332" r:id="rId811"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G333" r:id="rId812"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J333" r:id="rId813"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G334" r:id="rId814"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J334" r:id="rId815"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G335" r:id="rId816"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J335" r:id="rId817"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G336" r:id="rId818"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J336" r:id="rId819"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G337" r:id="rId820"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J337" r:id="rId821"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G338" r:id="rId822"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H338" r:id="rId823"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J338" r:id="rId824"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G339" r:id="rId825"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H339" r:id="rId826"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J339" r:id="rId827"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G340" r:id="rId828"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H340" r:id="rId829"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J340" r:id="rId830"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G341" r:id="rId831"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H341" r:id="rId832"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J341" r:id="rId833"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G342" r:id="rId834"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J342" r:id="rId835"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G343" r:id="rId836"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J343" r:id="rId837"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G344" r:id="rId838"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H344" r:id="rId839"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J344" r:id="rId840"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G345" r:id="rId841"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H345" r:id="rId842"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J345" r:id="rId843"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G346" r:id="rId844"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J346" r:id="rId845"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G347" r:id="rId846"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J347" r:id="rId847"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G348" r:id="rId848"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J348" r:id="rId849"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G349" r:id="rId850"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J349" r:id="rId851"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G350" r:id="rId852"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H350" r:id="rId853"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J350" r:id="rId854"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G351" r:id="rId855"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J351" r:id="rId856"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G352" r:id="rId857"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J352" r:id="rId858"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G353" r:id="rId859"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H353" r:id="rId860"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J353" r:id="rId861"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G354" r:id="rId862"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J354" r:id="rId863"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G355" r:id="rId864"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J355" r:id="rId865"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G356" r:id="rId866"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J356" r:id="rId867"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G357" r:id="rId868"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J357" r:id="rId869"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G358" r:id="rId870"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J358" r:id="rId871"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G359" r:id="rId872"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J359" r:id="rId873"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G360" r:id="rId874"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J360" r:id="rId875"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G361" r:id="rId876"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H361" r:id="rId877"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J361" r:id="rId878"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G362" r:id="rId879"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J362" r:id="rId880"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G363" r:id="rId881"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J363" r:id="rId882"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G364" r:id="rId883"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J364" r:id="rId884"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G365" r:id="rId885"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J365" r:id="rId886"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G366" r:id="rId887"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J366" r:id="rId888"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G367" r:id="rId889"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J367" r:id="rId890"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G368" r:id="rId891"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J368" r:id="rId892"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G369" r:id="rId893"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J369" r:id="rId894"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G370" r:id="rId895"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J370" r:id="rId896"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G371" r:id="rId897"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J371" r:id="rId898"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G372" r:id="rId899"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J372" r:id="rId900"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G373" r:id="rId901"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J373" r:id="rId902"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G374" r:id="rId903"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H374" r:id="rId904"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J374" r:id="rId905"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G375" r:id="rId906"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J375" r:id="rId907"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G376" r:id="rId908"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J376" r:id="rId909"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G377" r:id="rId910"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J377" r:id="rId911"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G378" r:id="rId912"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J378" r:id="rId913"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G379" r:id="rId914"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J379" r:id="rId915"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G380" r:id="rId916"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H380" r:id="rId917"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J380" r:id="rId918"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G381" r:id="rId919"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J381" r:id="rId920"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G382" r:id="rId921"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J382" r:id="rId922"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G383" r:id="rId923"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J383" r:id="rId924"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G384" r:id="rId925"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H384" r:id="rId926"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J384" r:id="rId927"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G385" r:id="rId928"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J385" r:id="rId929"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G386" r:id="rId930"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J386" r:id="rId931"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G387" r:id="rId932"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J387" r:id="rId933"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G388" r:id="rId934"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J388" r:id="rId935"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G389" r:id="rId936"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J389" r:id="rId937"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G390" r:id="rId938"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J390" r:id="rId939"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G391" r:id="rId940"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J391" r:id="rId941"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G392" r:id="rId942"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J392" r:id="rId943"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G393" r:id="rId944"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J393" r:id="rId945"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G394" r:id="rId946"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J394" r:id="rId947"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G395" r:id="rId948"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J395" r:id="rId949"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G396" r:id="rId950"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J396" r:id="rId951"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G397" r:id="rId952"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H397" r:id="rId953"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J397" r:id="rId954"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G398" r:id="rId955"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J398" r:id="rId956"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G399" r:id="rId957"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H399" r:id="rId958"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J399" r:id="rId959"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G400" r:id="rId960"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J400" r:id="rId961"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G401" r:id="rId962"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H401" r:id="rId963"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J401" r:id="rId964"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G402" r:id="rId965"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H402" r:id="rId966"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J402" r:id="rId967"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G403" r:id="rId968"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J403" r:id="rId969"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G404" r:id="rId970"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J404" r:id="rId971"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G405" r:id="rId972"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J405" r:id="rId973"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G406" r:id="rId974"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H406" r:id="rId975"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J406" r:id="rId976"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G407" r:id="rId977"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H407" r:id="rId978"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J407" r:id="rId979"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G408" r:id="rId980"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J408" r:id="rId981"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G409" r:id="rId982"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H409" r:id="rId983"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J409" r:id="rId984"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G410" r:id="rId985"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J410" r:id="rId986"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G411" r:id="rId987"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J411" r:id="rId988"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G412" r:id="rId989"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J412" r:id="rId990"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G413" r:id="rId991"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J413" r:id="rId992"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G414" r:id="rId993"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J414" r:id="rId994"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G415" r:id="rId995"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J415" r:id="rId996"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G416" r:id="rId997"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J416" r:id="rId998"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G417" r:id="rId999"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J417" r:id="rId1000"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G418" r:id="rId1001"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J418" r:id="rId1002"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G419" r:id="rId1003"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J419" r:id="rId1004"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G420" r:id="rId1005"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J420" r:id="rId1006"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G421" r:id="rId1007"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J421" r:id="rId1008"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G422" r:id="rId1009"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H422" r:id="rId1010"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J422" r:id="rId1011"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G423" r:id="rId1012"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H423" r:id="rId1013"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J423" r:id="rId1014"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G424" r:id="rId1015"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H424" r:id="rId1016"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J424" r:id="rId1017"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G425" r:id="rId1018"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H425" r:id="rId1019"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J425" r:id="rId1020"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G426" r:id="rId1021"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J426" r:id="rId1022"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G427" r:id="rId1023"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H427" r:id="rId1024"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J427" r:id="rId1025"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G428" r:id="rId1026"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J428" r:id="rId1027"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1025"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1028"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Split runs of statement titles merged into one heading block
Where the PDF shows separate centred headings, each title is split out with
the tool's Split block; wrapped titles stay whole. 137 headings, 22 sittings.
Changed sittings re-exported through Suggest hierarchy. New review zip 015-419.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M7thX74TYnsQKCuCTAUqbc
</commit_message>
<xml_diff>
--- a/12th Senate - audit results/All sittings in date order - finished or needs human check.xlsx
+++ b/12th Senate - audit results/All sittings in date order - finished or needs human check.xlsx
@@ -1445,7 +1445,7 @@
         </is>
       </c>
       <c r="K22" s="6" t="n">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="L22" s="6" t="n">
         <v>1</v>
@@ -1565,7 +1565,7 @@
         </is>
       </c>
       <c r="K24" s="6" t="n">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="L24" s="6" t="n">
         <v>3</v>
@@ -1625,7 +1625,7 @@
         </is>
       </c>
       <c r="K25" s="6" t="n">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="L25" s="6" t="n">
         <v>2</v>
@@ -1745,7 +1745,7 @@
         </is>
       </c>
       <c r="K27" s="6" t="n">
-        <v>189</v>
+        <v>198</v>
       </c>
       <c r="L27" s="6" t="n"/>
       <c r="M27" s="6" t="n"/>
@@ -2551,7 +2551,7 @@
         </is>
       </c>
       <c r="K41" s="6" t="n">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="L41" s="6" t="n">
         <v>7</v>
@@ -2611,7 +2611,7 @@
         </is>
       </c>
       <c r="K42" s="6" t="n">
-        <v>215</v>
+        <v>231</v>
       </c>
       <c r="L42" s="6" t="n"/>
       <c r="M42" s="6" t="n"/>
@@ -2675,7 +2675,7 @@
         </is>
       </c>
       <c r="K43" s="6" t="n">
-        <v>215</v>
+        <v>231</v>
       </c>
       <c r="L43" s="6" t="n"/>
       <c r="M43" s="6" t="n"/>
@@ -2729,7 +2729,7 @@
         </is>
       </c>
       <c r="K44" s="6" t="n">
-        <v>331</v>
+        <v>352</v>
       </c>
       <c r="L44" s="6" t="n"/>
       <c r="M44" s="6" t="n"/>
@@ -2955,7 +2955,7 @@
         </is>
       </c>
       <c r="K48" s="6" t="n">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="L48" s="6" t="n"/>
       <c r="M48" s="6" t="n"/>
@@ -3017,7 +3017,7 @@
         </is>
       </c>
       <c r="K49" s="6" t="n">
-        <v>701</v>
+        <v>704</v>
       </c>
       <c r="L49" s="6" t="n"/>
       <c r="M49" s="6" t="n"/>
@@ -3125,7 +3125,7 @@
         </is>
       </c>
       <c r="K51" s="6" t="n">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="L51" s="6" t="n"/>
       <c r="M51" s="6" t="n"/>
@@ -3181,7 +3181,7 @@
         </is>
       </c>
       <c r="K52" s="6" t="n">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="L52" s="6" t="n">
         <v>1</v>
@@ -3241,7 +3241,7 @@
         </is>
       </c>
       <c r="K53" s="6" t="n">
-        <v>274</v>
+        <v>284</v>
       </c>
       <c r="L53" s="6" t="n"/>
       <c r="M53" s="6" t="n">
@@ -3351,7 +3351,7 @@
         </is>
       </c>
       <c r="K55" s="6" t="n">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="L55" s="6" t="n">
         <v>4</v>
@@ -4035,7 +4035,7 @@
         </is>
       </c>
       <c r="K67" s="6" t="n">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="L67" s="6" t="n"/>
       <c r="M67" s="6" t="n">
@@ -4095,7 +4095,7 @@
         </is>
       </c>
       <c r="K68" s="6" t="n">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="L68" s="6" t="n"/>
       <c r="M68" s="6" t="n">
@@ -5065,7 +5065,7 @@
         </is>
       </c>
       <c r="K85" s="6" t="n">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="L85" s="6" t="n"/>
       <c r="M85" s="6" t="n"/>
@@ -18491,7 +18491,7 @@
         </is>
       </c>
       <c r="K327" s="6" t="n">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="L327" s="6" t="n"/>
       <c r="M327" s="6" t="n"/>
@@ -20337,7 +20337,7 @@
         </is>
       </c>
       <c r="K361" s="6" t="n">
-        <v>925</v>
+        <v>926</v>
       </c>
       <c r="L361" s="6" t="n"/>
       <c r="M361" s="6" t="n">
@@ -20599,7 +20599,7 @@
         </is>
       </c>
       <c r="K366" s="6" t="n">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="L366" s="6" t="n"/>
       <c r="M366" s="6" t="n"/>
@@ -20911,7 +20911,7 @@
         </is>
       </c>
       <c r="K372" s="6" t="n">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="L372" s="6" t="n"/>
       <c r="M372" s="6" t="n"/>
@@ -23853,7 +23853,7 @@
         </is>
       </c>
       <c r="K427" s="6" t="n">
-        <v>1058</v>
+        <v>1059</v>
       </c>
       <c r="L427" s="6" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Split out spaced-bracket scenes and delete embedded page headers
- PDF scenes left inside speeches because Mzalendo writes '( Sen. X ... )'
  with spaces: matched ignoring spacing, capped at the PDF's count (55).
- 'Month d, yyyy SENATEDEBATES n' page headers inside speeches split out
  and deleted (22, 2018-02-13).
Changed sittings re-exported through Suggest hierarchy. New zip 021-419.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M7thX74TYnsQKCuCTAUqbc
</commit_message>
<xml_diff>
--- a/12th Senate - audit results/All sittings in date order - finished or needs human check.xlsx
+++ b/12th Senate - audit results/All sittings in date order - finished or needs human check.xlsx
@@ -1019,7 +1019,7 @@
         </is>
       </c>
       <c r="K15" s="6" t="n">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="L15" s="6" t="n"/>
       <c r="M15" s="6" t="n"/>
@@ -1131,7 +1131,7 @@
         </is>
       </c>
       <c r="K17" s="6" t="n">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="L17" s="6" t="n"/>
       <c r="M17" s="6" t="n"/>
@@ -1255,7 +1255,7 @@
         </is>
       </c>
       <c r="K19" s="6" t="n">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="L19" s="6" t="n">
         <v>1</v>
@@ -1317,7 +1317,7 @@
         </is>
       </c>
       <c r="K20" s="6" t="n">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="L20" s="6" t="n">
         <v>3</v>
@@ -1381,7 +1381,7 @@
         </is>
       </c>
       <c r="K21" s="6" t="n">
-        <v>391</v>
+        <v>397</v>
       </c>
       <c r="L21" s="6" t="n">
         <v>1</v>
@@ -1445,7 +1445,7 @@
         </is>
       </c>
       <c r="K22" s="6" t="n">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="L22" s="6" t="n">
         <v>1</v>
@@ -1801,7 +1801,7 @@
         </is>
       </c>
       <c r="K28" s="6" t="n">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="L28" s="6" t="n">
         <v>6</v>
@@ -1859,7 +1859,7 @@
         </is>
       </c>
       <c r="K29" s="6" t="n">
-        <v>52</v>
+        <v>93</v>
       </c>
       <c r="L29" s="6" t="n"/>
       <c r="M29" s="6" t="n">
@@ -1977,7 +1977,7 @@
         </is>
       </c>
       <c r="K31" s="6" t="n">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="L31" s="6" t="n"/>
       <c r="M31" s="6" t="n">
@@ -2033,7 +2033,7 @@
         </is>
       </c>
       <c r="K32" s="6" t="n">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="L32" s="6" t="n"/>
       <c r="M32" s="6" t="n"/>
@@ -2375,7 +2375,7 @@
         </is>
       </c>
       <c r="K38" s="6" t="n">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="L38" s="6" t="n">
         <v>9</v>
@@ -2493,7 +2493,7 @@
         </is>
       </c>
       <c r="K40" s="6" t="n">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="L40" s="6" t="n"/>
       <c r="M40" s="6" t="n"/>
@@ -2785,7 +2785,7 @@
         </is>
       </c>
       <c r="K45" s="6" t="n">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="L45" s="6" t="n">
         <v>5</v>
@@ -2841,7 +2841,7 @@
         </is>
       </c>
       <c r="K46" s="6" t="n">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="L46" s="6" t="n"/>
       <c r="M46" s="6" t="n"/>
@@ -2955,7 +2955,7 @@
         </is>
       </c>
       <c r="K48" s="6" t="n">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="L48" s="6" t="n"/>
       <c r="M48" s="6" t="n"/>
@@ -3351,7 +3351,7 @@
         </is>
       </c>
       <c r="K55" s="6" t="n">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="L55" s="6" t="n">
         <v>4</v>
@@ -3407,7 +3407,7 @@
         </is>
       </c>
       <c r="K56" s="6" t="n">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="L56" s="6" t="n"/>
       <c r="M56" s="6" t="n"/>
@@ -3677,7 +3677,7 @@
         </is>
       </c>
       <c r="K61" s="6" t="n">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="L61" s="6" t="n">
         <v>3</v>
@@ -4771,7 +4771,7 @@
         </is>
       </c>
       <c r="K80" s="6" t="n">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="L80" s="6" t="n"/>
       <c r="M80" s="6" t="n"/>
@@ -5229,7 +5229,7 @@
         </is>
       </c>
       <c r="K88" s="6" t="n">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="L88" s="6" t="n"/>
       <c r="M88" s="6" t="n"/>
@@ -5661,7 +5661,7 @@
         </is>
       </c>
       <c r="K96" s="6" t="n">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="L96" s="6" t="n">
         <v>4</v>
@@ -5723,7 +5723,7 @@
         </is>
       </c>
       <c r="K97" s="6" t="n">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="L97" s="6" t="n">
         <v>1</v>
@@ -6181,7 +6181,7 @@
         </is>
       </c>
       <c r="K105" s="6" t="n">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="L105" s="6" t="n"/>
       <c r="M105" s="6" t="n"/>
@@ -6551,7 +6551,7 @@
         </is>
       </c>
       <c r="K112" s="6" t="n">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="L112" s="6" t="n"/>
       <c r="M112" s="6" t="n"/>
@@ -6603,7 +6603,7 @@
         </is>
       </c>
       <c r="K113" s="6" t="n">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="L113" s="6" t="n"/>
       <c r="M113" s="6" t="n"/>
@@ -8979,7 +8979,7 @@
         </is>
       </c>
       <c r="K155" s="6" t="n">
-        <v>653</v>
+        <v>655</v>
       </c>
       <c r="L155" s="6" t="n"/>
       <c r="M155" s="6" t="n"/>
@@ -9255,7 +9255,7 @@
         </is>
       </c>
       <c r="K160" s="6" t="n">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="L160" s="6" t="n">
         <v>2</v>
@@ -11531,7 +11531,7 @@
         </is>
       </c>
       <c r="K201" s="6" t="n">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="L201" s="6" t="n"/>
       <c r="M201" s="6" t="n"/>
@@ -12837,7 +12837,7 @@
         </is>
       </c>
       <c r="K225" s="6" t="n">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="L225" s="6" t="n">
         <v>4</v>
@@ -13101,7 +13101,7 @@
         </is>
       </c>
       <c r="K230" s="6" t="n">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="L230" s="6" t="n"/>
       <c r="M230" s="6" t="n"/>
@@ -13477,7 +13477,7 @@
         </is>
       </c>
       <c r="K237" s="6" t="n">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="L237" s="6" t="n"/>
       <c r="M237" s="6" t="n"/>
@@ -14083,7 +14083,7 @@
         </is>
       </c>
       <c r="K248" s="6" t="n">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="L248" s="6" t="n"/>
       <c r="M248" s="6" t="n"/>
@@ -16125,7 +16125,7 @@
         </is>
       </c>
       <c r="K284" s="6" t="n">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="L284" s="6" t="n">
         <v>1</v>
@@ -17245,7 +17245,7 @@
         </is>
       </c>
       <c r="K304" s="6" t="n">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="L304" s="6" t="n"/>
       <c r="M304" s="6" t="n"/>
@@ -19143,7 +19143,7 @@
         </is>
       </c>
       <c r="K339" s="6" t="n">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="L339" s="6" t="n"/>
       <c r="M339" s="6" t="n"/>
@@ -20177,7 +20177,7 @@
         </is>
       </c>
       <c r="K358" s="6" t="n">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="L358" s="6" t="n"/>
       <c r="M358" s="6" t="n"/>
@@ -20547,7 +20547,7 @@
         </is>
       </c>
       <c r="K365" s="6" t="n">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="L365" s="6" t="n"/>
       <c r="M365" s="6" t="n"/>
@@ -20599,7 +20599,7 @@
         </is>
       </c>
       <c r="K366" s="6" t="n">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="L366" s="6" t="n"/>
       <c r="M366" s="6" t="n"/>
@@ -20807,7 +20807,7 @@
         </is>
       </c>
       <c r="K370" s="6" t="n">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="L370" s="6" t="n"/>
       <c r="M370" s="6" t="n"/>
@@ -20859,7 +20859,7 @@
         </is>
       </c>
       <c r="K371" s="6" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="L371" s="6" t="n"/>
       <c r="M371" s="6" t="n"/>
@@ -21173,7 +21173,7 @@
         </is>
       </c>
       <c r="K377" s="6" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="L377" s="6" t="n"/>
       <c r="M377" s="6" t="n"/>
@@ -21803,7 +21803,7 @@
         </is>
       </c>
       <c r="K389" s="6" t="n">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="L389" s="6" t="n"/>
       <c r="M389" s="6" t="n"/>
@@ -22103,7 +22103,7 @@
         </is>
       </c>
       <c r="K395" s="6" t="n">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="L395" s="6" t="n"/>
       <c r="M395" s="6" t="n"/>
@@ -22155,7 +22155,7 @@
         </is>
       </c>
       <c r="K396" s="6" t="n">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="L396" s="6" t="n"/>
       <c r="M396" s="6" t="n"/>

</xml_diff>

<commit_message>
Put numbered list items back into their speeches (2018-03-06 on)
The first pass split indented items like '(a) ...' / '(i) ...' out of
speeches as scenes. Recombined with the tool's Combine with next (703),
3 ambiguous ones flagged; changed sittings re-exported through Suggest
hierarchy. Sittings before 2018-03-06 left unchanged. New review zip.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M7thX74TYnsQKCuCTAUqbc
</commit_message>
<xml_diff>
--- a/12th Senate - audit results/All sittings in date order - finished or needs human check.xlsx
+++ b/12th Senate - audit results/All sittings in date order - finished or needs human check.xlsx
@@ -2375,7 +2375,7 @@
         </is>
       </c>
       <c r="K38" s="6" t="n">
-        <v>396</v>
+        <v>390</v>
       </c>
       <c r="L38" s="6" t="n">
         <v>9</v>
@@ -2841,7 +2841,7 @@
         </is>
       </c>
       <c r="K46" s="6" t="n">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="L46" s="6" t="n"/>
       <c r="M46" s="6" t="n"/>
@@ -2955,7 +2955,7 @@
         </is>
       </c>
       <c r="K48" s="6" t="n">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="L48" s="6" t="n"/>
       <c r="M48" s="6" t="n"/>
@@ -3017,7 +3017,7 @@
         </is>
       </c>
       <c r="K49" s="6" t="n">
-        <v>704</v>
+        <v>664</v>
       </c>
       <c r="L49" s="6" t="n"/>
       <c r="M49" s="6" t="n"/>
@@ -3241,7 +3241,7 @@
         </is>
       </c>
       <c r="K53" s="6" t="n">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="L53" s="6" t="n"/>
       <c r="M53" s="6" t="n">
@@ -3459,7 +3459,7 @@
         </is>
       </c>
       <c r="K57" s="6" t="n">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="L57" s="6" t="n"/>
       <c r="M57" s="6" t="n"/>
@@ -3619,7 +3619,7 @@
         </is>
       </c>
       <c r="K60" s="6" t="n">
-        <v>200</v>
+        <v>178</v>
       </c>
       <c r="L60" s="6" t="n"/>
       <c r="M60" s="6" t="n"/>
@@ -3737,7 +3737,7 @@
         </is>
       </c>
       <c r="K62" s="6" t="n">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="L62" s="6" t="n">
         <v>1</v>
@@ -3861,7 +3861,7 @@
         </is>
       </c>
       <c r="K64" s="6" t="n">
-        <v>345</v>
+        <v>339</v>
       </c>
       <c r="L64" s="6" t="n">
         <v>3</v>
@@ -3925,7 +3925,7 @@
         </is>
       </c>
       <c r="K65" s="6" t="n">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="L65" s="6" t="n"/>
       <c r="M65" s="6" t="n"/>
@@ -4035,7 +4035,7 @@
         </is>
       </c>
       <c r="K67" s="6" t="n">
-        <v>450</v>
+        <v>446</v>
       </c>
       <c r="L67" s="6" t="n"/>
       <c r="M67" s="6" t="n">
@@ -4095,7 +4095,7 @@
         </is>
       </c>
       <c r="K68" s="6" t="n">
-        <v>471</v>
+        <v>465</v>
       </c>
       <c r="L68" s="6" t="n"/>
       <c r="M68" s="6" t="n">
@@ -4151,7 +4151,7 @@
         </is>
       </c>
       <c r="K69" s="6" t="n">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="L69" s="6" t="n"/>
       <c r="M69" s="6" t="n"/>
@@ -4317,7 +4317,7 @@
         </is>
       </c>
       <c r="K72" s="6" t="n">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="L72" s="6" t="n"/>
       <c r="M72" s="6" t="n">
@@ -4375,7 +4375,7 @@
         </is>
       </c>
       <c r="K73" s="6" t="n">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="L73" s="6" t="n">
         <v>3</v>
@@ -4495,7 +4495,7 @@
         </is>
       </c>
       <c r="K75" s="6" t="n">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="L75" s="6" t="n"/>
       <c r="M75" s="6" t="n"/>
@@ -4713,7 +4713,7 @@
         </is>
       </c>
       <c r="K79" s="6" t="n">
-        <v>410</v>
+        <v>388</v>
       </c>
       <c r="L79" s="6" t="n"/>
       <c r="M79" s="6" t="n"/>
@@ -4771,7 +4771,7 @@
         </is>
       </c>
       <c r="K80" s="6" t="n">
-        <v>306</v>
+        <v>284</v>
       </c>
       <c r="L80" s="6" t="n"/>
       <c r="M80" s="6" t="n"/>
@@ -5011,7 +5011,7 @@
         </is>
       </c>
       <c r="K84" s="6" t="n">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="L84" s="6" t="n">
         <v>1</v>
@@ -5065,7 +5065,7 @@
         </is>
       </c>
       <c r="K85" s="6" t="n">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="L85" s="6" t="n"/>
       <c r="M85" s="6" t="n"/>
@@ -5229,7 +5229,7 @@
         </is>
       </c>
       <c r="K88" s="6" t="n">
-        <v>366</v>
+        <v>360</v>
       </c>
       <c r="L88" s="6" t="n"/>
       <c r="M88" s="6" t="n"/>
@@ -5505,7 +5505,7 @@
         </is>
       </c>
       <c r="K93" s="6" t="n">
-        <v>460</v>
+        <v>454</v>
       </c>
       <c r="L93" s="6" t="n">
         <v>14</v>
@@ -5557,7 +5557,7 @@
         </is>
       </c>
       <c r="K94" s="6" t="n">
-        <v>323</v>
+        <v>317</v>
       </c>
       <c r="L94" s="6" t="n"/>
       <c r="M94" s="6" t="n"/>
@@ -5605,7 +5605,7 @@
         </is>
       </c>
       <c r="K95" s="6" t="n">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="L95" s="6" t="n"/>
       <c r="M95" s="6" t="n"/>
@@ -5661,7 +5661,7 @@
         </is>
       </c>
       <c r="K96" s="6" t="n">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="L96" s="6" t="n">
         <v>4</v>
@@ -5785,7 +5785,7 @@
         </is>
       </c>
       <c r="K98" s="6" t="n">
-        <v>256</v>
+        <v>246</v>
       </c>
       <c r="L98" s="6" t="n"/>
       <c r="M98" s="6" t="n"/>
@@ -5839,7 +5839,7 @@
         </is>
       </c>
       <c r="K99" s="6" t="n">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="L99" s="6" t="n"/>
       <c r="M99" s="6" t="n"/>
@@ -5895,7 +5895,7 @@
         </is>
       </c>
       <c r="K100" s="6" t="n">
-        <v>372</v>
+        <v>366</v>
       </c>
       <c r="L100" s="6" t="n">
         <v>6</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="K102" s="6" t="n">
-        <v>446</v>
+        <v>422</v>
       </c>
       <c r="L102" s="6" t="n"/>
       <c r="M102" s="6" t="n"/>
@@ -6129,7 +6129,7 @@
         </is>
       </c>
       <c r="K104" s="6" t="n">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="L104" s="6" t="n"/>
       <c r="M104" s="6" t="n"/>
@@ -6181,7 +6181,7 @@
         </is>
       </c>
       <c r="K105" s="6" t="n">
-        <v>552</v>
+        <v>516</v>
       </c>
       <c r="L105" s="6" t="n"/>
       <c r="M105" s="6" t="n"/>
@@ -6233,7 +6233,7 @@
         </is>
       </c>
       <c r="K106" s="6" t="n">
-        <v>234</v>
+        <v>222</v>
       </c>
       <c r="L106" s="6" t="n"/>
       <c r="M106" s="6" t="n"/>
@@ -6285,7 +6285,7 @@
         </is>
       </c>
       <c r="K107" s="6" t="n">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="L107" s="6" t="n"/>
       <c r="M107" s="6" t="n"/>
@@ -6337,7 +6337,7 @@
         </is>
       </c>
       <c r="K108" s="6" t="n">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="L108" s="6" t="n"/>
       <c r="M108" s="6" t="n"/>
@@ -6389,7 +6389,7 @@
         </is>
       </c>
       <c r="K109" s="6" t="n">
-        <v>196</v>
+        <v>160</v>
       </c>
       <c r="L109" s="6" t="n"/>
       <c r="M109" s="6" t="n"/>
@@ -6499,7 +6499,7 @@
         </is>
       </c>
       <c r="K111" s="6" t="n">
-        <v>370</v>
+        <v>364</v>
       </c>
       <c r="L111" s="6" t="n"/>
       <c r="M111" s="6" t="n"/>
@@ -6551,7 +6551,7 @@
         </is>
       </c>
       <c r="K112" s="6" t="n">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="L112" s="6" t="n"/>
       <c r="M112" s="6" t="n"/>
@@ -6603,7 +6603,7 @@
         </is>
       </c>
       <c r="K113" s="6" t="n">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="L113" s="6" t="n"/>
       <c r="M113" s="6" t="n"/>
@@ -6659,7 +6659,7 @@
         </is>
       </c>
       <c r="K114" s="6" t="n">
-        <v>244</v>
+        <v>228</v>
       </c>
       <c r="L114" s="6" t="n"/>
       <c r="M114" s="6" t="n">
@@ -6719,7 +6719,7 @@
         </is>
       </c>
       <c r="K115" s="6" t="n">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="L115" s="6" t="n"/>
       <c r="M115" s="6" t="n"/>
@@ -6783,7 +6783,7 @@
         </is>
       </c>
       <c r="K116" s="6" t="n">
-        <v>349</v>
+        <v>341</v>
       </c>
       <c r="L116" s="6" t="n"/>
       <c r="M116" s="6" t="n"/>
@@ -6899,7 +6899,7 @@
         </is>
       </c>
       <c r="K118" s="6" t="n">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="L118" s="6" t="n"/>
       <c r="M118" s="6" t="n"/>
@@ -6951,7 +6951,7 @@
         </is>
       </c>
       <c r="K119" s="6" t="n">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="L119" s="6" t="n"/>
       <c r="M119" s="6" t="n"/>
@@ -7007,7 +7007,7 @@
         </is>
       </c>
       <c r="K120" s="6" t="n">
-        <v>421</v>
+        <v>411</v>
       </c>
       <c r="L120" s="6" t="n"/>
       <c r="M120" s="6" t="n">
@@ -7065,7 +7065,7 @@
         </is>
       </c>
       <c r="K121" s="6" t="n">
-        <v>397</v>
+        <v>393</v>
       </c>
       <c r="L121" s="6" t="n">
         <v>6</v>
@@ -7173,7 +7173,7 @@
         </is>
       </c>
       <c r="K123" s="6" t="n">
-        <v>1574</v>
+        <v>1469</v>
       </c>
       <c r="L123" s="6" t="n"/>
       <c r="M123" s="6" t="n"/>
@@ -7229,7 +7229,7 @@
         </is>
       </c>
       <c r="K124" s="6" t="n">
-        <v>837</v>
+        <v>812</v>
       </c>
       <c r="L124" s="6" t="n"/>
       <c r="M124" s="6" t="n">
@@ -7407,7 +7407,7 @@
         </is>
       </c>
       <c r="K127" s="6" t="n">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="L127" s="6" t="n"/>
       <c r="M127" s="6" t="n">
@@ -7517,7 +7517,7 @@
         </is>
       </c>
       <c r="K129" s="6" t="n">
-        <v>438</v>
+        <v>432</v>
       </c>
       <c r="L129" s="6" t="n">
         <v>16</v>
@@ -7639,7 +7639,7 @@
         </is>
       </c>
       <c r="K131" s="6" t="n">
-        <v>440</v>
+        <v>430</v>
       </c>
       <c r="L131" s="6" t="n"/>
       <c r="M131" s="6" t="n"/>
@@ -7693,7 +7693,7 @@
         </is>
       </c>
       <c r="K132" s="6" t="n">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="L132" s="6" t="n"/>
       <c r="M132" s="6" t="n"/>
@@ -7745,7 +7745,7 @@
         </is>
       </c>
       <c r="K133" s="6" t="n">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="L133" s="6" t="n"/>
       <c r="M133" s="6" t="n"/>
@@ -7853,7 +7853,7 @@
         </is>
       </c>
       <c r="K135" s="6" t="n">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="L135" s="6" t="n"/>
       <c r="M135" s="6" t="n"/>
@@ -7973,7 +7973,7 @@
         </is>
       </c>
       <c r="K137" s="6" t="n">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="L137" s="6" t="n"/>
       <c r="M137" s="6" t="n"/>
@@ -8133,7 +8133,7 @@
         </is>
       </c>
       <c r="K140" s="6" t="n">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="L140" s="6" t="n">
         <v>1</v>
@@ -8195,7 +8195,7 @@
         </is>
       </c>
       <c r="K141" s="6" t="n">
-        <v>243</v>
+        <v>225</v>
       </c>
       <c r="L141" s="6" t="n">
         <v>5</v>
@@ -8481,7 +8481,7 @@
         </is>
       </c>
       <c r="K146" s="6" t="n">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="L146" s="6" t="n"/>
       <c r="M146" s="6" t="n">
@@ -8583,7 +8583,7 @@
         </is>
       </c>
       <c r="K148" s="6" t="n">
-        <v>234</v>
+        <v>204</v>
       </c>
       <c r="L148" s="6" t="n"/>
       <c r="M148" s="6" t="n"/>
@@ -8695,7 +8695,7 @@
         </is>
       </c>
       <c r="K150" s="6" t="n">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="L150" s="6" t="n"/>
       <c r="M150" s="6" t="n"/>
@@ -8747,7 +8747,7 @@
         </is>
       </c>
       <c r="K151" s="6" t="n">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="L151" s="6" t="n"/>
       <c r="M151" s="6" t="n"/>
@@ -8861,7 +8861,7 @@
         </is>
       </c>
       <c r="K153" s="6" t="n">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="L153" s="6" t="n">
         <v>1</v>
@@ -8979,7 +8979,7 @@
         </is>
       </c>
       <c r="K155" s="6" t="n">
-        <v>655</v>
+        <v>564</v>
       </c>
       <c r="L155" s="6" t="n"/>
       <c r="M155" s="6" t="n"/>
@@ -9035,7 +9035,7 @@
         </is>
       </c>
       <c r="K156" s="6" t="n">
-        <v>375</v>
+        <v>351</v>
       </c>
       <c r="L156" s="6" t="n"/>
       <c r="M156" s="6" t="n"/>
@@ -9141,7 +9141,7 @@
         </is>
       </c>
       <c r="K158" s="6" t="n">
-        <v>288</v>
+        <v>272</v>
       </c>
       <c r="L158" s="6" t="n"/>
       <c r="M158" s="6" t="n"/>
@@ -9197,7 +9197,7 @@
         </is>
       </c>
       <c r="K159" s="6" t="n">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="L159" s="6" t="n"/>
       <c r="M159" s="6" t="n">
@@ -9255,7 +9255,7 @@
         </is>
       </c>
       <c r="K160" s="6" t="n">
-        <v>683</v>
+        <v>675</v>
       </c>
       <c r="L160" s="6" t="n">
         <v>2</v>
@@ -9292,7 +9292,7 @@
         </is>
       </c>
       <c r="F161" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G161" s="9" t="inlineStr">
         <is>
@@ -9315,7 +9315,7 @@
         </is>
       </c>
       <c r="K161" s="6" t="n">
-        <v>582</v>
+        <v>557</v>
       </c>
       <c r="L161" s="6" t="n"/>
       <c r="M161" s="6" t="n">
@@ -9326,7 +9326,9 @@
       </c>
       <c r="O161" s="6" t="n"/>
       <c r="P161" s="6" t="n"/>
-      <c r="Q161" s="6" t="n"/>
+      <c r="Q161" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="R161" s="10" t="inlineStr"/>
     </row>
     <row r="162">
@@ -9375,7 +9377,7 @@
         </is>
       </c>
       <c r="K162" s="6" t="n">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="L162" s="6" t="n"/>
       <c r="M162" s="6" t="n">
@@ -9485,7 +9487,7 @@
         </is>
       </c>
       <c r="K164" s="6" t="n">
-        <v>270</v>
+        <v>258</v>
       </c>
       <c r="L164" s="6" t="n">
         <v>14</v>
@@ -9763,7 +9765,7 @@
         </is>
       </c>
       <c r="K169" s="6" t="n">
-        <v>752</v>
+        <v>677</v>
       </c>
       <c r="L169" s="6" t="n"/>
       <c r="M169" s="6" t="n">
@@ -9993,7 +9995,7 @@
         </is>
       </c>
       <c r="K173" s="6" t="n">
-        <v>417</v>
+        <v>404</v>
       </c>
       <c r="L173" s="6" t="n">
         <v>4</v>
@@ -10113,7 +10115,7 @@
         </is>
       </c>
       <c r="K175" s="6" t="n">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="L175" s="6" t="n">
         <v>1</v>
@@ -10231,7 +10233,7 @@
         </is>
       </c>
       <c r="K177" s="6" t="n">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="L177" s="6" t="n"/>
       <c r="M177" s="6" t="n"/>
@@ -10287,7 +10289,7 @@
         </is>
       </c>
       <c r="K178" s="6" t="n">
-        <v>431</v>
+        <v>427</v>
       </c>
       <c r="L178" s="6" t="n"/>
       <c r="M178" s="6" t="n"/>
@@ -10561,7 +10563,7 @@
         </is>
       </c>
       <c r="K183" s="6" t="n">
-        <v>1236</v>
+        <v>1234</v>
       </c>
       <c r="L183" s="6" t="n"/>
       <c r="M183" s="6" t="n"/>
@@ -10665,7 +10667,7 @@
         </is>
       </c>
       <c r="K185" s="6" t="n">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="L185" s="6" t="n"/>
       <c r="M185" s="6" t="n"/>
@@ -10995,7 +10997,7 @@
         </is>
       </c>
       <c r="K191" s="6" t="n">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="L191" s="6" t="n"/>
       <c r="M191" s="6" t="n"/>
@@ -11159,7 +11161,7 @@
         </is>
       </c>
       <c r="K194" s="6" t="n">
-        <v>341</v>
+        <v>335</v>
       </c>
       <c r="L194" s="6" t="n"/>
       <c r="M194" s="6" t="n"/>
@@ -11687,7 +11689,7 @@
         </is>
       </c>
       <c r="K204" s="6" t="n">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="L204" s="6" t="n"/>
       <c r="M204" s="6" t="n"/>
@@ -11791,7 +11793,7 @@
         </is>
       </c>
       <c r="K206" s="6" t="n">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="L206" s="6" t="n"/>
       <c r="M206" s="6" t="n"/>
@@ -11847,7 +11849,7 @@
         </is>
       </c>
       <c r="K207" s="6" t="n">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="L207" s="6" t="n">
         <v>4</v>
@@ -12071,7 +12073,7 @@
         </is>
       </c>
       <c r="K211" s="6" t="n">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="L211" s="6" t="n"/>
       <c r="M211" s="6" t="n"/>
@@ -12123,7 +12125,7 @@
         </is>
       </c>
       <c r="K212" s="6" t="n">
-        <v>307</v>
+        <v>297</v>
       </c>
       <c r="L212" s="6" t="n"/>
       <c r="M212" s="6" t="n"/>
@@ -12279,7 +12281,7 @@
         </is>
       </c>
       <c r="K215" s="6" t="n">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="L215" s="6" t="n"/>
       <c r="M215" s="6" t="n"/>
@@ -12445,7 +12447,7 @@
         </is>
       </c>
       <c r="K218" s="6" t="n">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="L218" s="6" t="n"/>
       <c r="M218" s="6" t="n"/>
@@ -12781,7 +12783,7 @@
         </is>
       </c>
       <c r="K224" s="6" t="n">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="L224" s="6" t="n"/>
       <c r="M224" s="6" t="n"/>
@@ -12837,7 +12839,7 @@
         </is>
       </c>
       <c r="K225" s="6" t="n">
-        <v>420</v>
+        <v>416</v>
       </c>
       <c r="L225" s="6" t="n">
         <v>4</v>
@@ -12945,7 +12947,7 @@
         </is>
       </c>
       <c r="K227" s="6" t="n">
-        <v>224</v>
+        <v>214</v>
       </c>
       <c r="L227" s="6" t="n"/>
       <c r="M227" s="6" t="n"/>
@@ -13049,7 +13051,7 @@
         </is>
       </c>
       <c r="K229" s="6" t="n">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="L229" s="6" t="n"/>
       <c r="M229" s="6" t="n"/>
@@ -13315,7 +13317,7 @@
         </is>
       </c>
       <c r="K234" s="6" t="n">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="L234" s="6" t="n"/>
       <c r="M234" s="6" t="n"/>
@@ -13423,7 +13425,7 @@
         </is>
       </c>
       <c r="K236" s="6" t="n">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="L236" s="6" t="n"/>
       <c r="M236" s="6" t="n">
@@ -13477,7 +13479,7 @@
         </is>
       </c>
       <c r="K237" s="6" t="n">
-        <v>368</v>
+        <v>362</v>
       </c>
       <c r="L237" s="6" t="n"/>
       <c r="M237" s="6" t="n"/>
@@ -13585,7 +13587,7 @@
         </is>
       </c>
       <c r="K239" s="6" t="n">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="L239" s="6" t="n">
         <v>14</v>
@@ -13813,7 +13815,7 @@
         </is>
       </c>
       <c r="K243" s="6" t="n">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="L243" s="6" t="n"/>
       <c r="M243" s="6" t="n"/>
@@ -13869,7 +13871,7 @@
         </is>
       </c>
       <c r="K244" s="6" t="n">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="L244" s="6" t="n"/>
       <c r="M244" s="6" t="n"/>
@@ -14031,7 +14033,7 @@
         </is>
       </c>
       <c r="K247" s="6" t="n">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="L247" s="6" t="n"/>
       <c r="M247" s="6" t="n"/>
@@ -14083,7 +14085,7 @@
         </is>
       </c>
       <c r="K248" s="6" t="n">
-        <v>577</v>
+        <v>555</v>
       </c>
       <c r="L248" s="6" t="n"/>
       <c r="M248" s="6" t="n"/>
@@ -14139,7 +14141,7 @@
         </is>
       </c>
       <c r="K249" s="6" t="n">
-        <v>574</v>
+        <v>555</v>
       </c>
       <c r="L249" s="6" t="n">
         <v>4</v>
@@ -14251,7 +14253,7 @@
         </is>
       </c>
       <c r="K251" s="6" t="n">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="L251" s="6" t="n"/>
       <c r="M251" s="6" t="n"/>
@@ -14305,7 +14307,7 @@
         </is>
       </c>
       <c r="K252" s="6" t="n">
-        <v>293</v>
+        <v>283</v>
       </c>
       <c r="L252" s="6" t="n"/>
       <c r="M252" s="6" t="n"/>
@@ -14357,7 +14359,7 @@
         </is>
       </c>
       <c r="K253" s="6" t="n">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="L253" s="6" t="n"/>
       <c r="M253" s="6" t="n"/>
@@ -14637,7 +14639,7 @@
         </is>
       </c>
       <c r="K258" s="6" t="n">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="L258" s="6" t="n"/>
       <c r="M258" s="6" t="n"/>
@@ -14695,7 +14697,7 @@
         </is>
       </c>
       <c r="K259" s="6" t="n">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="L259" s="6" t="n"/>
       <c r="M259" s="6" t="n">
@@ -14753,7 +14755,7 @@
         </is>
       </c>
       <c r="K260" s="6" t="n">
-        <v>471</v>
+        <v>463</v>
       </c>
       <c r="L260" s="6" t="n"/>
       <c r="M260" s="6" t="n"/>
@@ -14811,7 +14813,7 @@
         </is>
       </c>
       <c r="K261" s="6" t="n">
-        <v>471</v>
+        <v>467</v>
       </c>
       <c r="L261" s="6" t="n"/>
       <c r="M261" s="6" t="n"/>
@@ -15051,7 +15053,7 @@
         </is>
       </c>
       <c r="K265" s="6" t="n">
-        <v>387</v>
+        <v>383</v>
       </c>
       <c r="L265" s="6" t="n"/>
       <c r="M265" s="6" t="n"/>
@@ -15217,7 +15219,7 @@
         </is>
       </c>
       <c r="K268" s="6" t="n">
-        <v>570</v>
+        <v>566</v>
       </c>
       <c r="L268" s="6" t="n">
         <v>2</v>
@@ -15511,7 +15513,7 @@
         </is>
       </c>
       <c r="K273" s="6" t="n">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="L273" s="6" t="n"/>
       <c r="M273" s="6" t="n"/>
@@ -15905,7 +15907,7 @@
         </is>
       </c>
       <c r="K280" s="6" t="n">
-        <v>176</v>
+        <v>166</v>
       </c>
       <c r="L280" s="6" t="n"/>
       <c r="M280" s="6" t="n"/>
@@ -16015,7 +16017,7 @@
         </is>
       </c>
       <c r="K282" s="6" t="n">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="L282" s="6" t="n"/>
       <c r="M282" s="6" t="n"/>
@@ -16125,7 +16127,7 @@
         </is>
       </c>
       <c r="K284" s="6" t="n">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="L284" s="6" t="n">
         <v>1</v>
@@ -16442,7 +16444,7 @@
         </is>
       </c>
       <c r="F290" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G290" s="9" t="inlineStr">
         <is>
@@ -16465,7 +16467,7 @@
         </is>
       </c>
       <c r="K290" s="6" t="n">
-        <v>1510</v>
+        <v>1506</v>
       </c>
       <c r="L290" s="6" t="n">
         <v>8</v>
@@ -16478,7 +16480,9 @@
       </c>
       <c r="O290" s="6" t="n"/>
       <c r="P290" s="6" t="n"/>
-      <c r="Q290" s="6" t="n"/>
+      <c r="Q290" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="R290" s="10" t="inlineStr"/>
     </row>
     <row r="291">
@@ -16527,7 +16531,7 @@
         </is>
       </c>
       <c r="K291" s="6" t="n">
-        <v>536</v>
+        <v>526</v>
       </c>
       <c r="L291" s="6" t="n"/>
       <c r="M291" s="6" t="n"/>
@@ -16587,7 +16591,7 @@
         </is>
       </c>
       <c r="K292" s="6" t="n">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="L292" s="6" t="n"/>
       <c r="M292" s="6" t="n"/>
@@ -16967,7 +16971,7 @@
         </is>
       </c>
       <c r="K299" s="6" t="n">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="L299" s="6" t="n"/>
       <c r="M299" s="6" t="n"/>
@@ -17245,7 +17249,7 @@
         </is>
       </c>
       <c r="K304" s="6" t="n">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="L304" s="6" t="n"/>
       <c r="M304" s="6" t="n"/>
@@ -17297,7 +17301,7 @@
         </is>
       </c>
       <c r="K305" s="6" t="n">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="L305" s="6" t="n"/>
       <c r="M305" s="6" t="n"/>
@@ -17729,7 +17733,7 @@
         </is>
       </c>
       <c r="K313" s="6" t="n">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="L313" s="6" t="n"/>
       <c r="M313" s="6" t="n"/>
@@ -17989,7 +17993,7 @@
         </is>
       </c>
       <c r="K318" s="6" t="n">
-        <v>355</v>
+        <v>345</v>
       </c>
       <c r="L318" s="6" t="n"/>
       <c r="M318" s="6" t="n"/>
@@ -18491,7 +18495,7 @@
         </is>
       </c>
       <c r="K327" s="6" t="n">
-        <v>638</v>
+        <v>630</v>
       </c>
       <c r="L327" s="6" t="n"/>
       <c r="M327" s="6" t="n"/>
@@ -18711,7 +18715,7 @@
         </is>
       </c>
       <c r="K331" s="6" t="n">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="L331" s="6" t="n"/>
       <c r="M331" s="6" t="n"/>
@@ -19079,7 +19083,7 @@
         </is>
       </c>
       <c r="K338" s="6" t="n">
-        <v>1100</v>
+        <v>984</v>
       </c>
       <c r="L338" s="6" t="n">
         <v>7</v>
@@ -19182,7 +19186,7 @@
         </is>
       </c>
       <c r="F340" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G340" s="9" t="inlineStr">
         <is>
@@ -19205,7 +19209,7 @@
         </is>
       </c>
       <c r="K340" s="6" t="n">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="L340" s="6" t="n"/>
       <c r="M340" s="6" t="n"/>
@@ -19213,7 +19217,7 @@
       <c r="O340" s="6" t="n"/>
       <c r="P340" s="6" t="n"/>
       <c r="Q340" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R340" s="10" t="inlineStr">
         <is>
@@ -19373,7 +19377,7 @@
         </is>
       </c>
       <c r="K343" s="6" t="n">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="L343" s="6" t="n"/>
       <c r="M343" s="6" t="n"/>
@@ -19487,7 +19491,7 @@
         </is>
       </c>
       <c r="K345" s="6" t="n">
-        <v>439</v>
+        <v>431</v>
       </c>
       <c r="L345" s="6" t="n"/>
       <c r="M345" s="6" t="n"/>
@@ -19863,7 +19867,7 @@
         </is>
       </c>
       <c r="K352" s="6" t="n">
-        <v>224</v>
+        <v>210</v>
       </c>
       <c r="L352" s="6" t="n"/>
       <c r="M352" s="6" t="n"/>
@@ -20073,7 +20077,7 @@
         </is>
       </c>
       <c r="K356" s="6" t="n">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="L356" s="6" t="n"/>
       <c r="M356" s="6" t="n"/>
@@ -20229,7 +20233,7 @@
         </is>
       </c>
       <c r="K359" s="6" t="n">
-        <v>178</v>
+        <v>166</v>
       </c>
       <c r="L359" s="6" t="n"/>
       <c r="M359" s="6" t="n"/>
@@ -20337,7 +20341,7 @@
         </is>
       </c>
       <c r="K361" s="6" t="n">
-        <v>926</v>
+        <v>916</v>
       </c>
       <c r="L361" s="6" t="n"/>
       <c r="M361" s="6" t="n">
@@ -20391,7 +20395,7 @@
         </is>
       </c>
       <c r="K362" s="6" t="n">
-        <v>334</v>
+        <v>328</v>
       </c>
       <c r="L362" s="6" t="n"/>
       <c r="M362" s="6" t="n"/>
@@ -20755,7 +20759,7 @@
         </is>
       </c>
       <c r="K369" s="6" t="n">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="L369" s="6" t="n"/>
       <c r="M369" s="6" t="n"/>
@@ -21015,7 +21019,7 @@
         </is>
       </c>
       <c r="K374" s="6" t="n">
-        <v>1286</v>
+        <v>1284</v>
       </c>
       <c r="L374" s="6" t="n"/>
       <c r="M374" s="6" t="n"/>
@@ -21173,7 +21177,7 @@
         </is>
       </c>
       <c r="K377" s="6" t="n">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="L377" s="6" t="n"/>
       <c r="M377" s="6" t="n"/>
@@ -21387,7 +21391,7 @@
         </is>
       </c>
       <c r="K381" s="6" t="n">
-        <v>279</v>
+        <v>267</v>
       </c>
       <c r="L381" s="6" t="n"/>
       <c r="M381" s="6" t="n"/>
@@ -21951,7 +21955,7 @@
         </is>
       </c>
       <c r="K392" s="6" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="L392" s="6" t="n"/>
       <c r="M392" s="6" t="n"/>
@@ -22003,7 +22007,7 @@
         </is>
       </c>
       <c r="K393" s="6" t="n">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="L393" s="6" t="n"/>
       <c r="M393" s="6" t="n"/>
@@ -22103,7 +22107,7 @@
         </is>
       </c>
       <c r="K395" s="6" t="n">
-        <v>357</v>
+        <v>353</v>
       </c>
       <c r="L395" s="6" t="n"/>
       <c r="M395" s="6" t="n"/>
@@ -22937,7 +22941,7 @@
         </is>
       </c>
       <c r="K410" s="6" t="n">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="L410" s="6" t="n"/>
       <c r="M410" s="6" t="n"/>
@@ -23093,7 +23097,7 @@
         </is>
       </c>
       <c r="K413" s="6" t="n">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="L413" s="6" t="n"/>
       <c r="M413" s="6" t="n"/>
@@ -23197,7 +23201,7 @@
         </is>
       </c>
       <c r="K415" s="6" t="n">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="L415" s="6" t="n"/>
       <c r="M415" s="6" t="n"/>
@@ -23301,7 +23305,7 @@
         </is>
       </c>
       <c r="K417" s="6" t="n">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="L417" s="6" t="n"/>
       <c r="M417" s="6" t="n"/>
@@ -23353,7 +23357,7 @@
         </is>
       </c>
       <c r="K418" s="6" t="n">
-        <v>280</v>
+        <v>273</v>
       </c>
       <c r="L418" s="6" t="n"/>
       <c r="M418" s="6" t="n"/>
@@ -23853,7 +23857,7 @@
         </is>
       </c>
       <c r="K427" s="6" t="n">
-        <v>1059</v>
+        <v>1051</v>
       </c>
       <c r="L427" s="6" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Keep dropped headings as deleted blocks instead of removing them
The hidden-heading fix had removed 29 misplaced audit-inserted headings.
Restored 25 (2018-03-06 on) as deleted blocks (original_label heading),
in place; hidden_headings.py now marks them deleted instead of dropping.
New review zip from 2018-03-13.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M7thX74TYnsQKCuCTAUqbc
</commit_message>
<xml_diff>
--- a/12th Senate - audit results/All sittings in date order - finished or needs human check.xlsx
+++ b/12th Senate - audit results/All sittings in date order - finished or needs human check.xlsx
@@ -2785,7 +2785,7 @@
         </is>
       </c>
       <c r="K45" s="6" t="n">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="L45" s="6" t="n">
         <v>5</v>
@@ -3181,7 +3181,7 @@
         </is>
       </c>
       <c r="K52" s="6" t="n">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="L52" s="6" t="n">
         <v>1</v>
@@ -3241,7 +3241,7 @@
         </is>
       </c>
       <c r="K53" s="6" t="n">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="L53" s="6" t="n"/>
       <c r="M53" s="6" t="n">
@@ -3351,7 +3351,7 @@
         </is>
       </c>
       <c r="K55" s="6" t="n">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="L55" s="6" t="n">
         <v>4</v>
@@ -3511,7 +3511,7 @@
         </is>
       </c>
       <c r="K58" s="6" t="n">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="L58" s="6" t="n"/>
       <c r="M58" s="6" t="n"/>
@@ -3861,7 +3861,7 @@
         </is>
       </c>
       <c r="K64" s="6" t="n">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="L64" s="6" t="n">
         <v>3</v>
@@ -4151,7 +4151,7 @@
         </is>
       </c>
       <c r="K69" s="6" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="L69" s="6" t="n"/>
       <c r="M69" s="6" t="n"/>
@@ -4261,7 +4261,7 @@
         </is>
       </c>
       <c r="K71" s="6" t="n">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="L71" s="6" t="n"/>
       <c r="M71" s="6" t="n"/>
@@ -4949,7 +4949,7 @@
         </is>
       </c>
       <c r="K83" s="6" t="n">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="L83" s="6" t="n">
         <v>3</v>
@@ -5121,7 +5121,7 @@
         </is>
       </c>
       <c r="K86" s="6" t="n">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="L86" s="6" t="n">
         <v>1</v>
@@ -5393,7 +5393,7 @@
         </is>
       </c>
       <c r="K91" s="6" t="n">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="L91" s="6" t="n"/>
       <c r="M91" s="6" t="n"/>
@@ -5723,7 +5723,7 @@
         </is>
       </c>
       <c r="K97" s="6" t="n">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="L97" s="6" t="n">
         <v>1</v>
@@ -5895,7 +5895,7 @@
         </is>
       </c>
       <c r="K100" s="6" t="n">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="L100" s="6" t="n">
         <v>6</v>
@@ -8133,7 +8133,7 @@
         </is>
       </c>
       <c r="K140" s="6" t="n">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="L140" s="6" t="n">
         <v>1</v>
@@ -9657,7 +9657,7 @@
         </is>
       </c>
       <c r="K167" s="6" t="n">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="L167" s="6" t="n"/>
       <c r="M167" s="6" t="n"/>
@@ -15053,7 +15053,7 @@
         </is>
       </c>
       <c r="K265" s="6" t="n">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="L265" s="6" t="n"/>
       <c r="M265" s="6" t="n"/>
@@ -15455,7 +15455,7 @@
         </is>
       </c>
       <c r="K272" s="6" t="n">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="L272" s="6" t="n">
         <v>9</v>
@@ -17411,7 +17411,7 @@
         </is>
       </c>
       <c r="K307" s="6" t="n">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="L307" s="6" t="n"/>
       <c r="M307" s="6" t="n"/>
@@ -19433,7 +19433,7 @@
         </is>
       </c>
       <c r="K344" s="6" t="n">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="L344" s="6" t="n"/>
       <c r="M344" s="6" t="n"/>

</xml_diff>

<commit_message>
Apply rules learned from Owen's 40 finished sittings (2018-05-09 on)
Tested against Owen's sittings 2017-12-05 to 2018-05-08 before applying:
speaker names restored (from text or the PDF's turn line), broken Division
tallies combined, bill numbers combined into title headings, heading scraps
combined into speeches. Two candidate rules dropped after testing.
Sittings up to 2018-05-08 unchanged. New review zip from 2018-05-09.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M7thX74TYnsQKCuCTAUqbc
</commit_message>
<xml_diff>
--- a/12th Senate - audit results/All sittings in date order - finished or needs human check.xlsx
+++ b/12th Senate - audit results/All sittings in date order - finished or needs human check.xlsx
@@ -3241,7 +3241,7 @@
         </is>
       </c>
       <c r="K53" s="6" t="n">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="L53" s="6" t="n"/>
       <c r="M53" s="6" t="n">
@@ -3295,7 +3295,7 @@
         </is>
       </c>
       <c r="K54" s="6" t="n">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="L54" s="6" t="n"/>
       <c r="M54" s="6" t="n"/>
@@ -3351,7 +3351,7 @@
         </is>
       </c>
       <c r="K55" s="6" t="n">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="L55" s="6" t="n">
         <v>4</v>
@@ -3407,7 +3407,7 @@
         </is>
       </c>
       <c r="K56" s="6" t="n">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="L56" s="6" t="n"/>
       <c r="M56" s="6" t="n"/>
@@ -3459,7 +3459,7 @@
         </is>
       </c>
       <c r="K57" s="6" t="n">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="L57" s="6" t="n"/>
       <c r="M57" s="6" t="n"/>
@@ -3677,7 +3677,7 @@
         </is>
       </c>
       <c r="K61" s="6" t="n">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="L61" s="6" t="n">
         <v>3</v>
@@ -3737,7 +3737,7 @@
         </is>
       </c>
       <c r="K62" s="6" t="n">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="L62" s="6" t="n">
         <v>1</v>
@@ -3861,7 +3861,7 @@
         </is>
       </c>
       <c r="K64" s="6" t="n">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="L64" s="6" t="n">
         <v>3</v>
@@ -3925,7 +3925,7 @@
         </is>
       </c>
       <c r="K65" s="6" t="n">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="L65" s="6" t="n"/>
       <c r="M65" s="6" t="n"/>
@@ -4035,7 +4035,7 @@
         </is>
       </c>
       <c r="K67" s="6" t="n">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="L67" s="6" t="n"/>
       <c r="M67" s="6" t="n">
@@ -4095,7 +4095,7 @@
         </is>
       </c>
       <c r="K68" s="6" t="n">
-        <v>465</v>
+        <v>453</v>
       </c>
       <c r="L68" s="6" t="n"/>
       <c r="M68" s="6" t="n">
@@ -4375,7 +4375,7 @@
         </is>
       </c>
       <c r="K73" s="6" t="n">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="L73" s="6" t="n">
         <v>3</v>
@@ -4551,7 +4551,7 @@
         </is>
       </c>
       <c r="K76" s="6" t="n">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="L76" s="6" t="n"/>
       <c r="M76" s="6" t="n"/>
@@ -4713,7 +4713,7 @@
         </is>
       </c>
       <c r="K79" s="6" t="n">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="L79" s="6" t="n"/>
       <c r="M79" s="6" t="n"/>
@@ -4829,7 +4829,7 @@
         </is>
       </c>
       <c r="K81" s="6" t="n">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="L81" s="6" t="n"/>
       <c r="M81" s="6" t="n"/>
@@ -5065,7 +5065,7 @@
         </is>
       </c>
       <c r="K85" s="6" t="n">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="L85" s="6" t="n"/>
       <c r="M85" s="6" t="n"/>
@@ -5229,7 +5229,7 @@
         </is>
       </c>
       <c r="K88" s="6" t="n">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="L88" s="6" t="n"/>
       <c r="M88" s="6" t="n"/>
@@ -5285,7 +5285,7 @@
         </is>
       </c>
       <c r="K89" s="6" t="n">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="L89" s="6" t="n">
         <v>5</v>
@@ -5341,7 +5341,7 @@
         </is>
       </c>
       <c r="K90" s="6" t="n">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="L90" s="6" t="n"/>
       <c r="M90" s="6" t="n"/>
@@ -5393,7 +5393,7 @@
         </is>
       </c>
       <c r="K91" s="6" t="n">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="L91" s="6" t="n"/>
       <c r="M91" s="6" t="n"/>
@@ -5449,7 +5449,7 @@
         </is>
       </c>
       <c r="K92" s="6" t="n">
-        <v>395</v>
+        <v>390</v>
       </c>
       <c r="L92" s="6" t="n">
         <v>15</v>
@@ -5723,7 +5723,7 @@
         </is>
       </c>
       <c r="K97" s="6" t="n">
-        <v>489</v>
+        <v>475</v>
       </c>
       <c r="L97" s="6" t="n">
         <v>1</v>
@@ -6129,7 +6129,7 @@
         </is>
       </c>
       <c r="K104" s="6" t="n">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="L104" s="6" t="n"/>
       <c r="M104" s="6" t="n"/>
@@ -6181,7 +6181,7 @@
         </is>
       </c>
       <c r="K105" s="6" t="n">
-        <v>516</v>
+        <v>504</v>
       </c>
       <c r="L105" s="6" t="n"/>
       <c r="M105" s="6" t="n"/>
@@ -6285,7 +6285,7 @@
         </is>
       </c>
       <c r="K107" s="6" t="n">
-        <v>314</v>
+        <v>305</v>
       </c>
       <c r="L107" s="6" t="n"/>
       <c r="M107" s="6" t="n"/>
@@ -6445,7 +6445,7 @@
         </is>
       </c>
       <c r="K110" s="6" t="n">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="L110" s="6" t="n"/>
       <c r="M110" s="6" t="n"/>
@@ -6603,7 +6603,7 @@
         </is>
       </c>
       <c r="K113" s="6" t="n">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="L113" s="6" t="n"/>
       <c r="M113" s="6" t="n"/>
@@ -6659,7 +6659,7 @@
         </is>
       </c>
       <c r="K114" s="6" t="n">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="L114" s="6" t="n"/>
       <c r="M114" s="6" t="n">
@@ -7173,7 +7173,7 @@
         </is>
       </c>
       <c r="K123" s="6" t="n">
-        <v>1469</v>
+        <v>1465</v>
       </c>
       <c r="L123" s="6" t="n"/>
       <c r="M123" s="6" t="n"/>
@@ -7229,7 +7229,7 @@
         </is>
       </c>
       <c r="K124" s="6" t="n">
-        <v>812</v>
+        <v>780</v>
       </c>
       <c r="L124" s="6" t="n"/>
       <c r="M124" s="6" t="n">
@@ -7349,7 +7349,7 @@
         </is>
       </c>
       <c r="K126" s="6" t="n">
-        <v>542</v>
+        <v>524</v>
       </c>
       <c r="L126" s="6" t="n"/>
       <c r="M126" s="6" t="n">
@@ -7461,7 +7461,7 @@
         </is>
       </c>
       <c r="K128" s="6" t="n">
-        <v>329</v>
+        <v>321</v>
       </c>
       <c r="L128" s="6" t="n"/>
       <c r="M128" s="6" t="n"/>
@@ -7517,7 +7517,7 @@
         </is>
       </c>
       <c r="K129" s="6" t="n">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="L129" s="6" t="n">
         <v>16</v>
@@ -7577,7 +7577,7 @@
         </is>
       </c>
       <c r="K130" s="6" t="n">
-        <v>489</v>
+        <v>481</v>
       </c>
       <c r="L130" s="6" t="n">
         <v>8</v>
@@ -7693,7 +7693,7 @@
         </is>
       </c>
       <c r="K132" s="6" t="n">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="L132" s="6" t="n"/>
       <c r="M132" s="6" t="n"/>
@@ -7745,7 +7745,7 @@
         </is>
       </c>
       <c r="K133" s="6" t="n">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="L133" s="6" t="n"/>
       <c r="M133" s="6" t="n"/>
@@ -7797,7 +7797,7 @@
         </is>
       </c>
       <c r="K134" s="6" t="n">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="L134" s="6" t="n"/>
       <c r="M134" s="6" t="n"/>
@@ -7973,7 +7973,7 @@
         </is>
       </c>
       <c r="K137" s="6" t="n">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="L137" s="6" t="n"/>
       <c r="M137" s="6" t="n"/>
@@ -8133,7 +8133,7 @@
         </is>
       </c>
       <c r="K140" s="6" t="n">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="L140" s="6" t="n">
         <v>1</v>
@@ -8369,7 +8369,7 @@
         </is>
       </c>
       <c r="K144" s="6" t="n">
-        <v>273</v>
+        <v>267</v>
       </c>
       <c r="L144" s="6" t="n"/>
       <c r="M144" s="6" t="n">
@@ -8425,7 +8425,7 @@
         </is>
       </c>
       <c r="K145" s="6" t="n">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="L145" s="6" t="n"/>
       <c r="M145" s="6" t="n"/>
@@ -8639,7 +8639,7 @@
         </is>
       </c>
       <c r="K149" s="6" t="n">
-        <v>472</v>
+        <v>447</v>
       </c>
       <c r="L149" s="6" t="n">
         <v>4</v>
@@ -8803,7 +8803,7 @@
         </is>
       </c>
       <c r="K152" s="6" t="n">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="L152" s="6" t="n"/>
       <c r="M152" s="6" t="n"/>
@@ -8979,7 +8979,7 @@
         </is>
       </c>
       <c r="K155" s="6" t="n">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="L155" s="6" t="n"/>
       <c r="M155" s="6" t="n"/>
@@ -9089,7 +9089,7 @@
         </is>
       </c>
       <c r="K157" s="6" t="n">
-        <v>619</v>
+        <v>583</v>
       </c>
       <c r="L157" s="6" t="n"/>
       <c r="M157" s="6" t="n"/>
@@ -9197,7 +9197,7 @@
         </is>
       </c>
       <c r="K159" s="6" t="n">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="L159" s="6" t="n"/>
       <c r="M159" s="6" t="n">
@@ -9255,7 +9255,7 @@
         </is>
       </c>
       <c r="K160" s="6" t="n">
-        <v>675</v>
+        <v>649</v>
       </c>
       <c r="L160" s="6" t="n">
         <v>2</v>
@@ -9315,7 +9315,7 @@
         </is>
       </c>
       <c r="K161" s="6" t="n">
-        <v>557</v>
+        <v>547</v>
       </c>
       <c r="L161" s="6" t="n"/>
       <c r="M161" s="6" t="n">
@@ -9599,7 +9599,7 @@
         </is>
       </c>
       <c r="K166" s="6" t="n">
-        <v>585</v>
+        <v>567</v>
       </c>
       <c r="L166" s="6" t="n">
         <v>8</v>
@@ -9765,7 +9765,7 @@
         </is>
       </c>
       <c r="K169" s="6" t="n">
-        <v>677</v>
+        <v>672</v>
       </c>
       <c r="L169" s="6" t="n"/>
       <c r="M169" s="6" t="n">
@@ -9883,7 +9883,7 @@
         </is>
       </c>
       <c r="K171" s="6" t="n">
-        <v>363</v>
+        <v>356</v>
       </c>
       <c r="L171" s="6" t="n">
         <v>6</v>
@@ -9939,7 +9939,7 @@
         </is>
       </c>
       <c r="K172" s="6" t="n">
-        <v>445</v>
+        <v>431</v>
       </c>
       <c r="L172" s="6" t="n"/>
       <c r="M172" s="6" t="n"/>
@@ -10115,7 +10115,7 @@
         </is>
       </c>
       <c r="K175" s="6" t="n">
-        <v>411</v>
+        <v>405</v>
       </c>
       <c r="L175" s="6" t="n">
         <v>1</v>
@@ -10289,7 +10289,7 @@
         </is>
       </c>
       <c r="K178" s="6" t="n">
-        <v>427</v>
+        <v>421</v>
       </c>
       <c r="L178" s="6" t="n"/>
       <c r="M178" s="6" t="n"/>
@@ -10563,7 +10563,7 @@
         </is>
       </c>
       <c r="K183" s="6" t="n">
-        <v>1234</v>
+        <v>1226</v>
       </c>
       <c r="L183" s="6" t="n"/>
       <c r="M183" s="6" t="n"/>
@@ -11053,7 +11053,7 @@
         </is>
       </c>
       <c r="K192" s="6" t="n">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="L192" s="6" t="n">
         <v>12</v>
@@ -11377,7 +11377,7 @@
         </is>
       </c>
       <c r="K198" s="6" t="n">
-        <v>399</v>
+        <v>381</v>
       </c>
       <c r="L198" s="6" t="n"/>
       <c r="M198" s="6" t="n"/>
@@ -11849,7 +11849,7 @@
         </is>
       </c>
       <c r="K207" s="6" t="n">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="L207" s="6" t="n">
         <v>4</v>
@@ -11963,7 +11963,7 @@
         </is>
       </c>
       <c r="K209" s="6" t="n">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="L209" s="6" t="n">
         <v>15</v>
@@ -12229,7 +12229,7 @@
         </is>
       </c>
       <c r="K214" s="6" t="n">
-        <v>342</v>
+        <v>333</v>
       </c>
       <c r="L214" s="6" t="n"/>
       <c r="M214" s="6" t="n"/>
@@ -12447,7 +12447,7 @@
         </is>
       </c>
       <c r="K218" s="6" t="n">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="L218" s="6" t="n"/>
       <c r="M218" s="6" t="n"/>
@@ -12895,7 +12895,7 @@
         </is>
       </c>
       <c r="K226" s="6" t="n">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="L226" s="6" t="n"/>
       <c r="M226" s="6" t="n"/>
@@ -13369,7 +13369,7 @@
         </is>
       </c>
       <c r="K235" s="6" t="n">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="L235" s="6" t="n"/>
       <c r="M235" s="6" t="n"/>
@@ -13425,7 +13425,7 @@
         </is>
       </c>
       <c r="K236" s="6" t="n">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="L236" s="6" t="n"/>
       <c r="M236" s="6" t="n">
@@ -13531,7 +13531,7 @@
         </is>
       </c>
       <c r="K238" s="6" t="n">
-        <v>379</v>
+        <v>375</v>
       </c>
       <c r="L238" s="6" t="n"/>
       <c r="M238" s="6" t="n"/>
@@ -14033,7 +14033,7 @@
         </is>
       </c>
       <c r="K247" s="6" t="n">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="L247" s="6" t="n"/>
       <c r="M247" s="6" t="n"/>
@@ -14085,7 +14085,7 @@
         </is>
       </c>
       <c r="K248" s="6" t="n">
-        <v>555</v>
+        <v>549</v>
       </c>
       <c r="L248" s="6" t="n"/>
       <c r="M248" s="6" t="n"/>
@@ -14415,7 +14415,7 @@
         </is>
       </c>
       <c r="K254" s="6" t="n">
-        <v>446</v>
+        <v>425</v>
       </c>
       <c r="L254" s="6" t="n">
         <v>1</v>
@@ -14697,7 +14697,7 @@
         </is>
       </c>
       <c r="K259" s="6" t="n">
-        <v>382</v>
+        <v>362</v>
       </c>
       <c r="L259" s="6" t="n"/>
       <c r="M259" s="6" t="n">
@@ -14755,7 +14755,7 @@
         </is>
       </c>
       <c r="K260" s="6" t="n">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="L260" s="6" t="n"/>
       <c r="M260" s="6" t="n"/>
@@ -15219,7 +15219,7 @@
         </is>
       </c>
       <c r="K268" s="6" t="n">
-        <v>566</v>
+        <v>560</v>
       </c>
       <c r="L268" s="6" t="n">
         <v>2</v>
@@ -15455,7 +15455,7 @@
         </is>
       </c>
       <c r="K272" s="6" t="n">
-        <v>491</v>
+        <v>487</v>
       </c>
       <c r="L272" s="6" t="n">
         <v>9</v>
@@ -15569,7 +15569,7 @@
         </is>
       </c>
       <c r="K274" s="6" t="n">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L274" s="6" t="n">
         <v>13</v>
@@ -15625,7 +15625,7 @@
         </is>
       </c>
       <c r="K275" s="6" t="n">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="L275" s="6" t="n"/>
       <c r="M275" s="6" t="n"/>
@@ -15677,7 +15677,7 @@
         </is>
       </c>
       <c r="K276" s="6" t="n">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="L276" s="6" t="n"/>
       <c r="M276" s="6" t="n"/>
@@ -15729,7 +15729,7 @@
         </is>
       </c>
       <c r="K277" s="6" t="n">
-        <v>326</v>
+        <v>320</v>
       </c>
       <c r="L277" s="6" t="n"/>
       <c r="M277" s="6" t="n"/>
@@ -16643,7 +16643,7 @@
         </is>
       </c>
       <c r="K293" s="6" t="n">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="L293" s="6" t="n"/>
       <c r="M293" s="6" t="n"/>
@@ -16865,7 +16865,7 @@
         </is>
       </c>
       <c r="K297" s="6" t="n">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="L297" s="6" t="n">
         <v>1</v>
@@ -17197,7 +17197,7 @@
         </is>
       </c>
       <c r="K303" s="6" t="n">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="L303" s="6" t="n"/>
       <c r="M303" s="6" t="n"/>
@@ -17467,7 +17467,7 @@
         </is>
       </c>
       <c r="K308" s="6" t="n">
-        <v>597</v>
+        <v>588</v>
       </c>
       <c r="L308" s="6" t="n">
         <v>5</v>
@@ -17525,7 +17525,7 @@
         </is>
       </c>
       <c r="K309" s="6" t="n">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="L309" s="6" t="n"/>
       <c r="M309" s="6" t="n"/>
@@ -18495,7 +18495,7 @@
         </is>
       </c>
       <c r="K327" s="6" t="n">
-        <v>630</v>
+        <v>610</v>
       </c>
       <c r="L327" s="6" t="n"/>
       <c r="M327" s="6" t="n"/>
@@ -18551,7 +18551,7 @@
         </is>
       </c>
       <c r="K328" s="6" t="n">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="L328" s="6" t="n"/>
       <c r="M328" s="6" t="n">
@@ -18663,7 +18663,7 @@
         </is>
       </c>
       <c r="K330" s="6" t="n">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="L330" s="6" t="n"/>
       <c r="M330" s="6" t="n"/>
@@ -18923,7 +18923,7 @@
         </is>
       </c>
       <c r="K335" s="6" t="n">
-        <v>384</v>
+        <v>379</v>
       </c>
       <c r="L335" s="6" t="n"/>
       <c r="M335" s="6" t="n"/>
@@ -19083,7 +19083,7 @@
         </is>
       </c>
       <c r="K338" s="6" t="n">
-        <v>984</v>
+        <v>968</v>
       </c>
       <c r="L338" s="6" t="n">
         <v>7</v>
@@ -19271,7 +19271,7 @@
         </is>
       </c>
       <c r="K341" s="6" t="n">
-        <v>622</v>
+        <v>587</v>
       </c>
       <c r="L341" s="6" t="n"/>
       <c r="M341" s="6" t="n">
@@ -19377,7 +19377,7 @@
         </is>
       </c>
       <c r="K343" s="6" t="n">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="L343" s="6" t="n"/>
       <c r="M343" s="6" t="n"/>
@@ -19433,7 +19433,7 @@
         </is>
       </c>
       <c r="K344" s="6" t="n">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="L344" s="6" t="n"/>
       <c r="M344" s="6" t="n"/>
@@ -19545,7 +19545,7 @@
         </is>
       </c>
       <c r="K346" s="6" t="n">
-        <v>547</v>
+        <v>529</v>
       </c>
       <c r="L346" s="6" t="n"/>
       <c r="M346" s="6" t="n"/>
@@ -20341,7 +20341,7 @@
         </is>
       </c>
       <c r="K361" s="6" t="n">
-        <v>916</v>
+        <v>877</v>
       </c>
       <c r="L361" s="6" t="n"/>
       <c r="M361" s="6" t="n">
@@ -20759,7 +20759,7 @@
         </is>
       </c>
       <c r="K369" s="6" t="n">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="L369" s="6" t="n"/>
       <c r="M369" s="6" t="n"/>
@@ -21019,7 +21019,7 @@
         </is>
       </c>
       <c r="K374" s="6" t="n">
-        <v>1284</v>
+        <v>1233</v>
       </c>
       <c r="L374" s="6" t="n"/>
       <c r="M374" s="6" t="n"/>
@@ -21229,7 +21229,7 @@
         </is>
       </c>
       <c r="K378" s="6" t="n">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="L378" s="6" t="n"/>
       <c r="M378" s="6" t="n"/>
@@ -21337,7 +21337,7 @@
         </is>
       </c>
       <c r="K380" s="6" t="n">
-        <v>306</v>
+        <v>297</v>
       </c>
       <c r="L380" s="6" t="n"/>
       <c r="M380" s="6" t="n">
@@ -21391,7 +21391,7 @@
         </is>
       </c>
       <c r="K381" s="6" t="n">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="L381" s="6" t="n"/>
       <c r="M381" s="6" t="n"/>
@@ -21807,7 +21807,7 @@
         </is>
       </c>
       <c r="K389" s="6" t="n">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="L389" s="6" t="n"/>
       <c r="M389" s="6" t="n"/>
@@ -21855,7 +21855,7 @@
         </is>
       </c>
       <c r="K390" s="6" t="n">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="L390" s="6" t="n"/>
       <c r="M390" s="6" t="n"/>
@@ -21903,7 +21903,7 @@
         </is>
       </c>
       <c r="K391" s="6" t="n">
-        <v>375</v>
+        <v>352</v>
       </c>
       <c r="L391" s="6" t="n"/>
       <c r="M391" s="6" t="n"/>
@@ -22107,7 +22107,7 @@
         </is>
       </c>
       <c r="K395" s="6" t="n">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="L395" s="6" t="n"/>
       <c r="M395" s="6" t="n"/>
@@ -22159,7 +22159,7 @@
         </is>
       </c>
       <c r="K396" s="6" t="n">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="L396" s="6" t="n"/>
       <c r="M396" s="6" t="n"/>
@@ -22385,7 +22385,7 @@
         </is>
       </c>
       <c r="K400" s="6" t="n">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="L400" s="6" t="n"/>
       <c r="M400" s="6" t="n"/>
@@ -22441,7 +22441,7 @@
         </is>
       </c>
       <c r="K401" s="6" t="n">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="L401" s="6" t="n"/>
       <c r="M401" s="6" t="n"/>
@@ -22499,7 +22499,7 @@
         </is>
       </c>
       <c r="K402" s="6" t="n">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="L402" s="6" t="n"/>
       <c r="M402" s="6" t="n"/>
@@ -22661,7 +22661,7 @@
         </is>
       </c>
       <c r="K405" s="6" t="n">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L405" s="6" t="n"/>
       <c r="M405" s="6" t="n"/>
@@ -22717,7 +22717,7 @@
         </is>
       </c>
       <c r="K406" s="6" t="n">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L406" s="6" t="n"/>
       <c r="M406" s="6" t="n"/>
@@ -22775,7 +22775,7 @@
         </is>
       </c>
       <c r="K407" s="6" t="n">
-        <v>364</v>
+        <v>360</v>
       </c>
       <c r="L407" s="6" t="n"/>
       <c r="M407" s="6" t="n">
@@ -22885,7 +22885,7 @@
         </is>
       </c>
       <c r="K409" s="6" t="n">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="L409" s="6" t="n">
         <v>15</v>
@@ -23045,7 +23045,7 @@
         </is>
       </c>
       <c r="K412" s="6" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="L412" s="6" t="n"/>
       <c r="M412" s="6" t="n"/>
@@ -23201,7 +23201,7 @@
         </is>
       </c>
       <c r="K415" s="6" t="n">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="L415" s="6" t="n"/>
       <c r="M415" s="6" t="n"/>
@@ -23509,7 +23509,7 @@
         </is>
       </c>
       <c r="K421" s="6" t="n">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="L421" s="6" t="n"/>
       <c r="M421" s="6" t="n"/>
@@ -23565,7 +23565,7 @@
         </is>
       </c>
       <c r="K422" s="6" t="n">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L422" s="6" t="n"/>
       <c r="M422" s="6" t="n"/>
@@ -23623,7 +23623,7 @@
         </is>
       </c>
       <c r="K423" s="6" t="n">
-        <v>683</v>
+        <v>657</v>
       </c>
       <c r="L423" s="6" t="n"/>
       <c r="M423" s="6" t="n">
@@ -23857,7 +23857,7 @@
         </is>
       </c>
       <c r="K427" s="6" t="n">
-        <v>1051</v>
+        <v>1024</v>
       </c>
       <c r="L427" s="6" t="n">
         <v>1</v>

</xml_diff>